<commit_message>
Add SCD Type 2 template + auto detection in ddl_generator
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D243EF-6A5A-4D1E-A2FD-3283F085FEEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD8173B1-7CC7-4860-854F-C4B51F5B927F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="72">
   <si>
     <t>Source_Name</t>
   </si>
@@ -112,9 +112,6 @@
   </si>
   <si>
     <t>Source_File_Mapping</t>
-  </si>
-  <si>
-    <t>raw/Brands</t>
   </si>
   <si>
     <t>raw/MDM</t>
@@ -264,6 +261,9 @@
   </si>
   <si>
     <t>bit</t>
+  </si>
+  <si>
+    <t>Is_Required</t>
   </si>
 </sst>
 </file>
@@ -729,16 +729,16 @@
         <v>23</v>
       </c>
       <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
         <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>28</v>
       </c>
       <c r="D2" t="s">
         <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F2">
         <v>0.1</v>
@@ -747,7 +747,7 @@
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -755,16 +755,16 @@
         <v>24</v>
       </c>
       <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
         <v>27</v>
-      </c>
-      <c r="C3" t="s">
-        <v>28</v>
       </c>
       <c r="D3" t="s">
         <v>24</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F3">
         <v>0.11</v>
@@ -773,7 +773,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -781,16 +781,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E4" t="s">
         <v>67</v>
-      </c>
-      <c r="E4" t="s">
-        <v>68</v>
       </c>
       <c r="F4" s="4">
         <v>1</v>
@@ -810,10 +810,10 @@
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -844,7 +844,7 @@
     <col min="5" max="5" width="23.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -861,21 +861,24 @@
         <v>6</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>14</v>
@@ -889,16 +892,19 @@
       <c r="G2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>14</v>
@@ -912,16 +918,19 @@
       <c r="G3" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>14</v>
@@ -935,16 +944,19 @@
       <c r="G4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>14</v>
@@ -958,16 +970,19 @@
       <c r="G5" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>14</v>
@@ -981,16 +996,19 @@
       <c r="G6" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>14</v>
@@ -1004,16 +1022,19 @@
       <c r="G7" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>14</v>
@@ -1027,8 +1048,11 @@
       <c r="G8" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1050,8 +1074,11 @@
       <c r="G9" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1065,7 +1092,7 @@
         <v>14</v>
       </c>
       <c r="E10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
@@ -1073,8 +1100,11 @@
       <c r="G10" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1088,7 +1118,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F11" t="b">
         <v>1</v>
@@ -1096,8 +1126,11 @@
       <c r="G11" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1111,7 +1144,7 @@
         <v>14</v>
       </c>
       <c r="E12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -1119,8 +1152,11 @@
       <c r="G12" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -1134,7 +1170,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -1142,8 +1178,11 @@
       <c r="G13" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1157,7 +1196,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
@@ -1165,8 +1204,11 @@
       <c r="G14" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -1177,10 +1219,10 @@
         <v>5</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F15" t="b">
         <v>0</v>
@@ -1188,8 +1230,11 @@
       <c r="G15" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -1203,7 +1248,7 @@
         <v>14</v>
       </c>
       <c r="E16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F16" t="b">
         <v>0</v>
@@ -1211,8 +1256,11 @@
       <c r="G16" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -1226,7 +1274,7 @@
         <v>14</v>
       </c>
       <c r="E17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F17" t="b">
         <v>0</v>
@@ -1234,8 +1282,11 @@
       <c r="G17" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -1249,7 +1300,7 @@
         <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F18" t="b">
         <v>0</v>
@@ -1257,8 +1308,11 @@
       <c r="G18" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -1272,7 +1326,7 @@
         <v>14</v>
       </c>
       <c r="E19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F19" t="b">
         <v>0</v>
@@ -1280,8 +1334,11 @@
       <c r="G19" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1295,7 +1352,7 @@
         <v>14</v>
       </c>
       <c r="E20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
@@ -1303,8 +1360,11 @@
       <c r="G20" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -1318,7 +1378,7 @@
         <v>14</v>
       </c>
       <c r="E21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F21" t="b">
         <v>0</v>
@@ -1326,16 +1386,19 @@
       <c r="G21" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>9</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>14</v>
@@ -1349,16 +1412,19 @@
       <c r="G22" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>9</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>14</v>
@@ -1372,40 +1438,46 @@
       <c r="G23" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>9</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C24" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" t="s">
-        <v>63</v>
-      </c>
       <c r="F24" t="b">
         <v>0</v>
       </c>
       <c r="G24" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B25" s="5"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>

</xml_diff>

<commit_message>
remove dydnamic creation dynamic creation od system sql objects
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD8173B1-7CC7-4860-854F-C4B51F5B927F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DBA736-AEDF-4CA6-B352-DA3929B67149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="75">
   <si>
     <t>Source_Name</t>
   </si>
@@ -264,6 +264,15 @@
   </si>
   <si>
     <t>Is_Required</t>
+  </si>
+  <si>
+    <t>SCD Type 2 Field</t>
+  </si>
+  <si>
+    <t>Is the column part of the PK</t>
+  </si>
+  <si>
+    <t>Is the column nullable</t>
   </si>
 </sst>
 </file>
@@ -334,7 +343,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -348,6 +357,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -835,7 +847,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C70B00-7E47-4939-BD03-7BD8F4F3F11B}">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr defaultColWidth="18.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" customWidth="1"/>
@@ -886,13 +898,13 @@
       <c r="E2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="b">
-        <v>0</v>
-      </c>
-      <c r="G2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" t="b">
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
         <v>1</v>
       </c>
     </row>
@@ -912,13 +924,13 @@
       <c r="E3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G3" t="b">
-        <v>0</v>
-      </c>
-      <c r="H3" t="b">
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
         <v>1</v>
       </c>
     </row>
@@ -938,13 +950,13 @@
       <c r="E4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F4" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4" t="b">
-        <v>0</v>
-      </c>
-      <c r="H4" t="b">
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
         <v>0</v>
       </c>
     </row>
@@ -964,13 +976,13 @@
       <c r="E5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5" t="b">
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
         <v>0</v>
       </c>
     </row>
@@ -990,13 +1002,13 @@
       <c r="E6" t="s">
         <v>19</v>
       </c>
-      <c r="F6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H6" t="b">
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>0</v>
       </c>
     </row>
@@ -1016,13 +1028,13 @@
       <c r="E7" t="s">
         <v>20</v>
       </c>
-      <c r="F7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G7" t="b">
-        <v>0</v>
-      </c>
-      <c r="H7" t="b">
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
         <v>0</v>
       </c>
     </row>
@@ -1042,13 +1054,13 @@
       <c r="E8" t="s">
         <v>21</v>
       </c>
-      <c r="F8" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H8" t="b">
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
         <v>0</v>
       </c>
     </row>
@@ -1068,13 +1080,13 @@
       <c r="E9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F9" t="b">
-        <v>0</v>
-      </c>
-      <c r="G9" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" t="b">
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
         <v>1</v>
       </c>
     </row>
@@ -1094,13 +1106,13 @@
       <c r="E10" t="s">
         <v>40</v>
       </c>
-      <c r="F10" t="b">
-        <v>1</v>
-      </c>
-      <c r="G10" t="b">
-        <v>0</v>
-      </c>
-      <c r="H10" t="b">
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
         <v>1</v>
       </c>
     </row>
@@ -1120,13 +1132,13 @@
       <c r="E11" t="s">
         <v>39</v>
       </c>
-      <c r="F11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" t="b">
-        <v>0</v>
-      </c>
-      <c r="H11" t="b">
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
         <v>1</v>
       </c>
     </row>
@@ -1146,13 +1158,13 @@
       <c r="E12" t="s">
         <v>41</v>
       </c>
-      <c r="F12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" t="b">
-        <v>0</v>
-      </c>
-      <c r="H12" t="b">
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
         <v>0</v>
       </c>
     </row>
@@ -1172,13 +1184,13 @@
       <c r="E13" t="s">
         <v>49</v>
       </c>
-      <c r="F13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" t="b">
-        <v>0</v>
-      </c>
-      <c r="H13" t="b">
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
         <v>1</v>
       </c>
     </row>
@@ -1198,13 +1210,13 @@
       <c r="E14" t="s">
         <v>47</v>
       </c>
-      <c r="F14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G14" t="b">
-        <v>0</v>
-      </c>
-      <c r="H14" t="b">
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
         <v>0</v>
       </c>
     </row>
@@ -1224,13 +1236,13 @@
       <c r="E15" t="s">
         <v>46</v>
       </c>
-      <c r="F15" t="b">
-        <v>0</v>
-      </c>
-      <c r="G15" t="b">
-        <v>0</v>
-      </c>
-      <c r="H15" t="b">
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
         <v>1</v>
       </c>
     </row>
@@ -1250,13 +1262,13 @@
       <c r="E16" t="s">
         <v>50</v>
       </c>
-      <c r="F16" t="b">
-        <v>0</v>
-      </c>
-      <c r="G16" t="b">
-        <v>0</v>
-      </c>
-      <c r="H16" t="b">
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
         <v>0</v>
       </c>
     </row>
@@ -1276,13 +1288,13 @@
       <c r="E17" t="s">
         <v>43</v>
       </c>
-      <c r="F17" t="b">
-        <v>0</v>
-      </c>
-      <c r="G17" t="b">
-        <v>1</v>
-      </c>
-      <c r="H17" t="b">
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
         <v>1</v>
       </c>
     </row>
@@ -1302,13 +1314,13 @@
       <c r="E18" t="s">
         <v>42</v>
       </c>
-      <c r="F18" t="b">
-        <v>0</v>
-      </c>
-      <c r="G18" t="b">
-        <v>1</v>
-      </c>
-      <c r="H18" t="b">
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
         <v>1</v>
       </c>
     </row>
@@ -1328,13 +1340,13 @@
       <c r="E19" t="s">
         <v>44</v>
       </c>
-      <c r="F19" t="b">
-        <v>0</v>
-      </c>
-      <c r="G19" t="b">
-        <v>0</v>
-      </c>
-      <c r="H19" t="b">
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
         <v>1</v>
       </c>
     </row>
@@ -1354,13 +1366,13 @@
       <c r="E20" t="s">
         <v>45</v>
       </c>
-      <c r="F20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G20" t="b">
-        <v>0</v>
-      </c>
-      <c r="H20" t="b">
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
         <v>1</v>
       </c>
     </row>
@@ -1380,116 +1392,194 @@
       <c r="E21" t="s">
         <v>48</v>
       </c>
-      <c r="F21" t="b">
-        <v>0</v>
-      </c>
-      <c r="G21" t="b">
-        <v>0</v>
-      </c>
-      <c r="H21" t="b">
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>9</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>32</v>
+        <v>24</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F22" t="b">
-        <v>0</v>
-      </c>
-      <c r="G22" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" t="b">
+        <v>70</v>
+      </c>
+      <c r="E22" t="s">
+        <v>72</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>9</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>60</v>
+        <v>24</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F23" t="b">
-        <v>0</v>
-      </c>
-      <c r="G23" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" t="b">
+        <v>70</v>
+      </c>
+      <c r="E23" t="s">
+        <v>73</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E24" t="s">
+        <v>74</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B25" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C27" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" t="s">
+      <c r="D27" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" t="s">
         <v>62</v>
       </c>
-      <c r="F24" t="b">
-        <v>0</v>
-      </c>
-      <c r="G24" t="b">
-        <v>0</v>
-      </c>
-      <c r="H24" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="5"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-    </row>
-    <row r="33" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B28" s="5"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
cleaned up .sql template where issue
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -343,7 +343,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -357,9 +357,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1406,10 +1403,10 @@
       <c r="A22" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="8" t="s">
         <v>68</v>
       </c>
       <c r="D22" s="3" t="s">
@@ -1432,10 +1429,10 @@
       <c r="A23" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="8" t="s">
         <v>69</v>
       </c>
       <c r="D23" s="3" t="s">
@@ -1458,10 +1455,10 @@
       <c r="A24" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="8" t="s">
         <v>71</v>
       </c>
       <c r="D24" s="3" t="s">

</xml_diff>

<commit_message>
Fixed config file issue for data paths
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DBA736-AEDF-4CA6-B352-DA3929B67149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39613892-6DAD-41A2-A71D-01D0D24DF8EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="74">
   <si>
     <t>Source_Name</t>
   </si>
@@ -232,9 +232,6 @@
   </si>
   <si>
     <t>Principals.xlsx</t>
-  </si>
-  <si>
-    <t>sheet1</t>
   </si>
   <si>
     <t>Sheet1</t>
@@ -796,10 +793,10 @@
         <v>64</v>
       </c>
       <c r="D4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" t="s">
         <v>66</v>
-      </c>
-      <c r="E4" t="s">
-        <v>67</v>
       </c>
       <c r="F4" s="4">
         <v>1</v>
@@ -870,13 +867,13 @@
         <v>6</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1228,7 +1225,7 @@
         <v>5</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E15" t="s">
         <v>46</v>
@@ -1404,16 +1401,16 @@
         <v>24</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -1430,16 +1427,16 @@
         <v>24</v>
       </c>
       <c r="B23" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>70</v>
-      </c>
       <c r="E23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1456,16 +1453,16 @@
         <v>24</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F24">
         <v>0</v>

</xml_diff>

<commit_message>
Unit testing updates, added DW_Table_Name and Merge_Proc_Name to Source_Imports
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39613892-6DAD-41A2-A71D-01D0D24DF8EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B71EBE-B327-49B6-A2D5-2A9F032747DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="86">
   <si>
     <t>Source_Name</t>
   </si>
@@ -270,6 +270,42 @@
   </si>
   <si>
     <t>Is the column nullable</t>
+  </si>
+  <si>
+    <t>DW_Table_Name</t>
+  </si>
+  <si>
+    <t>Merge_Proc_Name</t>
+  </si>
+  <si>
+    <t>[DW].[Dim_Brands]</t>
+  </si>
+  <si>
+    <t>[DW].[Dim_Principals]</t>
+  </si>
+  <si>
+    <t>[ETL].[Dim_Source_Imports]</t>
+  </si>
+  <si>
+    <t>[ETL].[Dim_Source_Imports_Mapping]</t>
+  </si>
+  <si>
+    <t>[DW].[SP_Merge_Dim_Brands]</t>
+  </si>
+  <si>
+    <t>[DW].[SP_Merge_Dim_Principals]</t>
+  </si>
+  <si>
+    <t>[ETL].[SP_Merge_Dim_Source_Imports]</t>
+  </si>
+  <si>
+    <t>[ETL].[SP_Merge_Dim_Source_Imports_Mapping]</t>
+  </si>
+  <si>
+    <t>Target Data Warehouse Dimension or fact name</t>
+  </si>
+  <si>
+    <t>ETL Phase 2 Stored Procedure</t>
   </si>
 </sst>
 </file>
@@ -691,7 +727,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{584572B9-381C-487F-864D-5B674FBBA046}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
@@ -701,10 +737,12 @@
     <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.28515625" customWidth="1"/>
     <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -729,8 +767,14 @@
       <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -755,8 +799,14 @@
       <c r="H2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -781,8 +831,14 @@
       <c r="H3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" t="s">
+        <v>79</v>
+      </c>
+      <c r="J3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -807,8 +863,14 @@
       <c r="H4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4" t="s">
+        <v>77</v>
+      </c>
+      <c r="J4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -832,6 +894,12 @@
       </c>
       <c r="H5" t="s">
         <v>8</v>
+      </c>
+      <c r="I5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J5" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -841,13 +909,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C70B00-7E47-4939-BD03-7BD8F4F3F11B}">
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr defaultColWidth="18.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" customWidth="1"/>
     <col min="2" max="2" width="27.85546875" customWidth="1"/>
     <col min="3" max="3" width="31.28515625" customWidth="1"/>
-    <col min="5" max="5" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1268,25 +1336,25 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="B17" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E17" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="F17">
         <v>0</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17">
         <v>1</v>
@@ -1294,25 +1362,25 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="B18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" t="s">
+        <v>75</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>42</v>
+        <v>85</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18">
         <v>1</v>
@@ -1323,22 +1391,22 @@
         <v>24</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19">
         <v>1</v>
@@ -1349,22 +1417,22 @@
         <v>24</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E20" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F20">
         <v>0</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -1375,16 +1443,16 @@
         <v>24</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E21" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1393,7 +1461,7 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1401,16 +1469,16 @@
         <v>24</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E22" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -1427,16 +1495,16 @@
         <v>24</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E23" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1445,7 +1513,7 @@
         <v>0</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1453,16 +1521,16 @@
         <v>24</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1476,25 +1544,25 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>9</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>32</v>
+        <v>24</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>68</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>15</v>
+        <v>69</v>
+      </c>
+      <c r="E25" t="s">
+        <v>72</v>
       </c>
       <c r="F25">
         <v>0</v>
       </c>
       <c r="G25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H25">
         <v>1</v>
@@ -1502,25 +1570,25 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>9</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>60</v>
+        <v>24</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>70</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>15</v>
+        <v>69</v>
+      </c>
+      <c r="E26" t="s">
+        <v>73</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H26">
         <v>1</v>
@@ -1531,49 +1599,101 @@
         <v>9</v>
       </c>
       <c r="B27" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+      <c r="H28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C29" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" t="s">
+      <c r="D29" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29" t="s">
         <v>62</v>
       </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
-      <c r="G27">
-        <v>0</v>
-      </c>
-      <c r="H27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B28" s="5"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B30" s="5"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Make DDL unit tests robust to whitespace and formatting differences
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B71EBE-B327-49B6-A2D5-2A9F032747DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BC9337F-DDE2-4649-867F-17AF6BDDB6E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="103">
   <si>
     <t>Source_Name</t>
   </si>
@@ -307,12 +307,63 @@
   <si>
     <t>ETL Phase 2 Stored Procedure</t>
   </si>
+  <si>
+    <t>Force_DDL_Generation</t>
+  </si>
+  <si>
+    <t>Wholesaler Code</t>
+  </si>
+  <si>
+    <t>Wholesaler Name</t>
+  </si>
+  <si>
+    <t>Wholesaler Address</t>
+  </si>
+  <si>
+    <t>Wholesaler City</t>
+  </si>
+  <si>
+    <t>Wholesaler Province</t>
+  </si>
+  <si>
+    <t>Wholesaler Country</t>
+  </si>
+  <si>
+    <t>Wholesalers</t>
+  </si>
+  <si>
+    <t>Wholesaler_Code</t>
+  </si>
+  <si>
+    <t>Wholesaler_Name</t>
+  </si>
+  <si>
+    <t>Wholesaler_Address</t>
+  </si>
+  <si>
+    <t>Wholesaler_City</t>
+  </si>
+  <si>
+    <t>Wholesaler_Province</t>
+  </si>
+  <si>
+    <t>Wholesaler_Country</t>
+  </si>
+  <si>
+    <t>VARCHAR(255)</t>
+  </si>
+  <si>
+    <t>Wholesalers.xlsx</t>
+  </si>
+  <si>
+    <t>ODS.Wholesalers</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -327,13 +378,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -374,9 +418,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -386,9 +430,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -727,7 +770,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{584572B9-381C-487F-864D-5B674FBBA046}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
@@ -742,7 +785,7 @@
     <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -773,8 +816,11 @@
       <c r="J1" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -805,8 +851,11 @@
       <c r="J2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -837,8 +886,11 @@
       <c r="J3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -869,8 +921,11 @@
       <c r="J4" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -900,6 +955,44 @@
       </c>
       <c r="J5" t="s">
         <v>80</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" t="s">
+        <v>102</v>
+      </c>
+      <c r="F6">
+        <v>1.2</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I6" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" t="s">
+        <v>80</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -948,7 +1041,7 @@
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -974,7 +1067,7 @@
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>52</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -1000,7 +1093,7 @@
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -1026,7 +1119,7 @@
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>54</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -1052,7 +1145,7 @@
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>55</v>
       </c>
       <c r="C6" t="s">
@@ -1078,7 +1171,7 @@
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C7" t="s">
@@ -1104,7 +1197,7 @@
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>57</v>
       </c>
       <c r="C8" t="s">
@@ -1390,10 +1483,10 @@
       <c r="A19" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="C19" s="8" t="s">
+      <c r="B19" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>0</v>
       </c>
       <c r="D19" s="3" t="s">
@@ -1416,10 +1509,10 @@
       <c r="A20" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="7" t="s">
         <v>11</v>
       </c>
       <c r="D20" s="3" t="s">
@@ -1442,10 +1535,10 @@
       <c r="A21" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="3" t="s">
@@ -1468,10 +1561,10 @@
       <c r="A22" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="7" t="s">
         <v>13</v>
       </c>
       <c r="D22" s="3" t="s">
@@ -1494,10 +1587,10 @@
       <c r="A23" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="7" t="s">
         <v>6</v>
       </c>
       <c r="D23" s="3" t="s">
@@ -1520,10 +1613,10 @@
       <c r="A24" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D24" s="3" t="s">
@@ -1546,10 +1639,10 @@
       <c r="A25" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>68</v>
       </c>
       <c r="D25" s="3" t="s">
@@ -1572,10 +1665,10 @@
       <c r="A26" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="7" t="s">
         <v>70</v>
       </c>
       <c r="D26" s="3" t="s">
@@ -1598,7 +1691,7 @@
       <c r="A27" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C27" s="3" t="s">
@@ -1624,10 +1717,10 @@
       <c r="A28" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>60</v>
       </c>
       <c r="D28" s="3" t="s">
@@ -1650,10 +1743,10 @@
       <c r="A29" t="s">
         <v>9</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>61</v>
       </c>
       <c r="D29" s="3" t="s">
@@ -1673,27 +1766,174 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B30" s="5"/>
+      <c r="A30" t="s">
+        <v>93</v>
+      </c>
+      <c r="B30" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" t="s">
+        <v>94</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30">
+        <v>1</v>
+      </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
+      <c r="A31" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" t="s">
+        <v>95</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>93</v>
+      </c>
+      <c r="B32" t="s">
+        <v>89</v>
+      </c>
+      <c r="C32" t="s">
+        <v>96</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33" t="s">
+        <v>90</v>
+      </c>
+      <c r="C33" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E33" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>93</v>
+      </c>
+      <c r="B34" t="s">
+        <v>91</v>
+      </c>
+      <c r="C34" t="s">
+        <v>98</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E34" t="s">
+        <v>20</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>93</v>
+      </c>
+      <c r="B35" t="s">
+        <v>92</v>
+      </c>
+      <c r="C35" t="s">
+        <v>99</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E35" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
DW DDL: add Row_Change_Reason to all dims, remove unnecessary temp cleanup, double-trim Target_Column. Still testing
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BC9337F-DDE2-4649-867F-17AF6BDDB6E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8521ABC6-6AC9-4291-A76A-694D3F7F21AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
@@ -69,9 +69,6 @@
     <t>Brands</t>
   </si>
   <si>
-    <t>ODS.Brands</t>
-  </si>
-  <si>
     <t>Source_Column</t>
   </si>
   <si>
@@ -123,12 +120,6 @@
     <t>ETL_Config.xlsx</t>
   </si>
   <si>
-    <t>ETL.Source_Imports</t>
-  </si>
-  <si>
-    <t>ETL.Source_File_Mapping</t>
-  </si>
-  <si>
     <t>List of flat file imports</t>
   </si>
   <si>
@@ -235,9 +226,6 @@
   </si>
   <si>
     <t>Sheet1</t>
-  </si>
-  <si>
-    <t>ODS.Principals</t>
   </si>
   <si>
     <r>
@@ -356,7 +344,19 @@
     <t>Wholesalers.xlsx</t>
   </si>
   <si>
-    <t>ODS.Wholesalers</t>
+    <t>[ODS].[Principals]</t>
+  </si>
+  <si>
+    <t>[ODS].[Brands]</t>
+  </si>
+  <si>
+    <t>[ODS].[Wholesalers]</t>
+  </si>
+  <si>
+    <t>[ETL].[Source_Imports]</t>
+  </si>
+  <si>
+    <t>[ETL].[Source_File_Mapping]</t>
   </si>
 </sst>
 </file>
@@ -802,7 +802,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
@@ -811,30 +811,30 @@
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
         <v>26</v>
       </c>
-      <c r="C2" t="s">
-        <v>27</v>
-      </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>101</v>
       </c>
       <c r="F2">
         <v>0.1</v>
@@ -843,13 +843,13 @@
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="I2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J2" t="s">
         <v>78</v>
-      </c>
-      <c r="J2" t="s">
-        <v>82</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -857,19 +857,19 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
         <v>26</v>
       </c>
-      <c r="C3" t="s">
-        <v>27</v>
-      </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>102</v>
       </c>
       <c r="F3">
         <v>0.11</v>
@@ -878,13 +878,13 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I3" t="s">
+        <v>75</v>
+      </c>
+      <c r="J3" t="s">
         <v>79</v>
-      </c>
-      <c r="J3" t="s">
-        <v>83</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -895,16 +895,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>66</v>
+        <v>98</v>
       </c>
       <c r="F4" s="4">
         <v>1</v>
@@ -916,10 +916,10 @@
         <v>8</v>
       </c>
       <c r="I4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J4" t="s">
         <v>77</v>
-      </c>
-      <c r="J4" t="s">
-        <v>81</v>
       </c>
       <c r="K4">
         <v>1</v>
@@ -930,16 +930,16 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="F5" s="4">
         <v>1.1000000000000001</v>
@@ -951,10 +951,10 @@
         <v>8</v>
       </c>
       <c r="I5" t="s">
+        <v>72</v>
+      </c>
+      <c r="J5" t="s">
         <v>76</v>
-      </c>
-      <c r="J5" t="s">
-        <v>80</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -962,19 +962,19 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F6">
         <v>1.2</v>
@@ -986,10 +986,10 @@
         <v>8</v>
       </c>
       <c r="I6" t="s">
+        <v>72</v>
+      </c>
+      <c r="J6" t="s">
         <v>76</v>
-      </c>
-      <c r="J6" t="s">
-        <v>80</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -1016,25 +1016,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1042,16 +1042,16 @@
         <v>7</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1068,16 +1068,16 @@
         <v>7</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -1094,16 +1094,16 @@
         <v>7</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -1120,16 +1120,16 @@
         <v>7</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -1146,16 +1146,16 @@
         <v>7</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -1172,16 +1172,16 @@
         <v>7</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -1198,16 +1198,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -1221,7 +1221,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
         <v>0</v>
@@ -1230,10 +1230,10 @@
         <v>0</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -1247,7 +1247,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
         <v>1</v>
@@ -1256,10 +1256,10 @@
         <v>1</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -1273,7 +1273,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" t="s">
         <v>2</v>
@@ -1282,10 +1282,10 @@
         <v>2</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -1299,7 +1299,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s">
         <v>3</v>
@@ -1308,10 +1308,10 @@
         <v>3</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -1325,7 +1325,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
         <v>4</v>
@@ -1334,10 +1334,10 @@
         <v>4</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -1351,19 +1351,19 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E14" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -1377,7 +1377,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
         <v>5</v>
@@ -1386,10 +1386,10 @@
         <v>5</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E15" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -1403,7 +1403,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" t="s">
         <v>6</v>
@@ -1412,10 +1412,10 @@
         <v>6</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E16" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -1429,19 +1429,19 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C17" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1455,19 +1455,19 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C18" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E18" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -1481,7 +1481,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>0</v>
@@ -1490,10 +1490,10 @@
         <v>0</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -1507,19 +1507,19 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E20" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -1533,19 +1533,19 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E21" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1559,19 +1559,19 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E22" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -1585,7 +1585,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>6</v>
@@ -1594,10 +1594,10 @@
         <v>6</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E23" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1611,19 +1611,19 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" t="s">
         <v>67</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E24" t="s">
-        <v>71</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1637,19 +1637,19 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E25" t="s">
         <v>68</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E25" t="s">
-        <v>72</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1663,19 +1663,19 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D26" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E26" t="s">
         <v>69</v>
-      </c>
-      <c r="E26" t="s">
-        <v>73</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1692,16 +1692,16 @@
         <v>9</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D27" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1718,16 +1718,16 @@
         <v>9</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D28" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="F28">
         <v>0</v>
@@ -1744,16 +1744,16 @@
         <v>9</v>
       </c>
       <c r="B29" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" t="s">
         <v>59</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E29" t="s">
-        <v>62</v>
       </c>
       <c r="F29">
         <v>0</v>
@@ -1767,19 +1767,19 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B30" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C30" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F30">
         <v>0</v>
@@ -1793,19 +1793,19 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B31" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C31" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F31">
         <v>0</v>
@@ -1819,19 +1819,19 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B32" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C32" t="s">
+        <v>92</v>
+      </c>
+      <c r="D32" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D32" s="3" t="s">
-        <v>100</v>
-      </c>
       <c r="E32" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F32">
         <v>0</v>
@@ -1845,19 +1845,19 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>89</v>
+      </c>
+      <c r="B33" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" t="s">
         <v>93</v>
       </c>
-      <c r="B33" t="s">
-        <v>90</v>
-      </c>
-      <c r="C33" t="s">
-        <v>97</v>
-      </c>
       <c r="D33" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E33" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F33">
         <v>0</v>
@@ -1871,19 +1871,19 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C34" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -1897,19 +1897,19 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B35" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C35" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F35">
         <v>0</v>

</xml_diff>

<commit_message>
Restore force DDL generation logic + silence Pandas warning
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8521ABC6-6AC9-4291-A76A-694D3F7F21AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6209A94F-EEAE-4809-BFA5-85DD40B68FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
@@ -1132,7 +1132,7 @@
         <v>17</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1158,7 +1158,7 @@
         <v>18</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6">
         <v>0</v>

</xml_diff>

<commit_message>
Troubleshooting source file forats csv
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6209A94F-EEAE-4809-BFA5-85DD40B68FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9537CAB-0B2D-4300-885E-BE46FC1D97BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="180">
   <si>
     <t>Source_Name</t>
   </si>
@@ -278,12 +278,6 @@
     <t>[ETL].[Dim_Source_Imports_Mapping]</t>
   </si>
   <si>
-    <t>[DW].[SP_Merge_Dim_Brands]</t>
-  </si>
-  <si>
-    <t>[DW].[SP_Merge_Dim_Principals]</t>
-  </si>
-  <si>
     <t>[ETL].[SP_Merge_Dim_Source_Imports]</t>
   </si>
   <si>
@@ -357,6 +351,243 @@
   </si>
   <si>
     <t>[ETL].[Source_File_Mapping]</t>
+  </si>
+  <si>
+    <t>Product code</t>
+  </si>
+  <si>
+    <t>Product Name</t>
+  </si>
+  <si>
+    <t>Product Barcode</t>
+  </si>
+  <si>
+    <t>Principal ID</t>
+  </si>
+  <si>
+    <t>Brand ID</t>
+  </si>
+  <si>
+    <t>Product Department</t>
+  </si>
+  <si>
+    <t>Product Category</t>
+  </si>
+  <si>
+    <t>Product Segment</t>
+  </si>
+  <si>
+    <t>Product Sub-segment</t>
+  </si>
+  <si>
+    <t>Product Packaging type</t>
+  </si>
+  <si>
+    <t>Units of measure</t>
+  </si>
+  <si>
+    <t>Product Volume</t>
+  </si>
+  <si>
+    <t>Product Variant</t>
+  </si>
+  <si>
+    <t>Product Case size</t>
+  </si>
+  <si>
+    <t>Product Nappi code</t>
+  </si>
+  <si>
+    <t>Product Schedule</t>
+  </si>
+  <si>
+    <t>Product_Code</t>
+  </si>
+  <si>
+    <t>Product_Name</t>
+  </si>
+  <si>
+    <t>Product_Barcode</t>
+  </si>
+  <si>
+    <t>Product_Department</t>
+  </si>
+  <si>
+    <t>Product_Category</t>
+  </si>
+  <si>
+    <t>Product_Segment</t>
+  </si>
+  <si>
+    <t>Product_Sub_Segment</t>
+  </si>
+  <si>
+    <t>Product_Packaging_Type</t>
+  </si>
+  <si>
+    <t>Unit_Of_Measure</t>
+  </si>
+  <si>
+    <t>Product_Volume</t>
+  </si>
+  <si>
+    <t>Product_Variant</t>
+  </si>
+  <si>
+    <t>Product_Case_Size</t>
+  </si>
+  <si>
+    <t>Product_Nappi_Code</t>
+  </si>
+  <si>
+    <t>Product_Schedule</t>
+  </si>
+  <si>
+    <t>Products</t>
+  </si>
+  <si>
+    <t>raw/MDM/Products</t>
+  </si>
+  <si>
+    <t>*.xlsx</t>
+  </si>
+  <si>
+    <t>[ODS].[Products]</t>
+  </si>
+  <si>
+    <t>medium dimension, multiple files</t>
+  </si>
+  <si>
+    <t>[DW].[Dim_Wholesalers]</t>
+  </si>
+  <si>
+    <t>[DW].[Dim_Products]</t>
+  </si>
+  <si>
+    <t>[ETL].[SP_Merge_Dim_Principals]</t>
+  </si>
+  <si>
+    <t>[ETL].[SP_Merge_Dim_Brands]</t>
+  </si>
+  <si>
+    <t>[ETL].[SP_Merge_Dim_Wholesalers]</t>
+  </si>
+  <si>
+    <t>[ETL].[SP_Merge_Dim_Products]</t>
+  </si>
+  <si>
+    <t>Places</t>
+  </si>
+  <si>
+    <t>raw/MDM/Places</t>
+  </si>
+  <si>
+    <t>[ODS].[Places]</t>
+  </si>
+  <si>
+    <t>[DW].[Dim_Places]</t>
+  </si>
+  <si>
+    <t>[ETL].[SP_Merge_Dim_Places]</t>
+  </si>
+  <si>
+    <t>Place code</t>
+  </si>
+  <si>
+    <t>Place Name</t>
+  </si>
+  <si>
+    <t>Place Category</t>
+  </si>
+  <si>
+    <t>Place Sub-category</t>
+  </si>
+  <si>
+    <t>Place Chain</t>
+  </si>
+  <si>
+    <t>Place Address</t>
+  </si>
+  <si>
+    <t>Place City</t>
+  </si>
+  <si>
+    <t>Place Province</t>
+  </si>
+  <si>
+    <t>Place Country</t>
+  </si>
+  <si>
+    <t>Place Latitude</t>
+  </si>
+  <si>
+    <t>Place Longitude</t>
+  </si>
+  <si>
+    <t>Place Contact Number</t>
+  </si>
+  <si>
+    <t>Place Contact Name</t>
+  </si>
+  <si>
+    <t>Place Contact Title</t>
+  </si>
+  <si>
+    <t>Place Contact Email</t>
+  </si>
+  <si>
+    <t>Place Website</t>
+  </si>
+  <si>
+    <t>Place_Code</t>
+  </si>
+  <si>
+    <t>Place_Name</t>
+  </si>
+  <si>
+    <t>Place_Category</t>
+  </si>
+  <si>
+    <t>Place_Sub_Category</t>
+  </si>
+  <si>
+    <t>Place_Chain</t>
+  </si>
+  <si>
+    <t>Place_Address</t>
+  </si>
+  <si>
+    <t>Place_City</t>
+  </si>
+  <si>
+    <t>Place_Province</t>
+  </si>
+  <si>
+    <t>Place_Country</t>
+  </si>
+  <si>
+    <t>Place_Latitude</t>
+  </si>
+  <si>
+    <t>Place_Longitude</t>
+  </si>
+  <si>
+    <t>Place_Contact_Number</t>
+  </si>
+  <si>
+    <t>Place_Contact_Name</t>
+  </si>
+  <si>
+    <t>Place_Contact_Title</t>
+  </si>
+  <si>
+    <t>Place_Contact_Email</t>
+  </si>
+  <si>
+    <t>Place_Website</t>
+  </si>
+  <si>
+    <t>Is_Type2_Attribute</t>
   </si>
 </sst>
 </file>
@@ -399,12 +630,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -420,7 +657,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -435,6 +672,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -770,19 +1010,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{584572B9-381C-487F-864D-5B674FBBA046}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.28515625" customWidth="1"/>
     <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.140625" customWidth="1"/>
+    <col min="10" max="10" width="43.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -817,7 +1057,7 @@
         <v>71</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -834,7 +1074,7 @@
         <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F2">
         <v>0.1</v>
@@ -849,7 +1089,7 @@
         <v>74</v>
       </c>
       <c r="J2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -869,7 +1109,7 @@
         <v>23</v>
       </c>
       <c r="E3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F3">
         <v>0.11</v>
@@ -884,7 +1124,7 @@
         <v>75</v>
       </c>
       <c r="J3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -904,7 +1144,7 @@
         <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F4" s="4">
         <v>1</v>
@@ -919,10 +1159,10 @@
         <v>73</v>
       </c>
       <c r="J4" t="s">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -939,7 +1179,7 @@
         <v>62</v>
       </c>
       <c r="E5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F5" s="4">
         <v>1.1000000000000001</v>
@@ -954,45 +1194,115 @@
         <v>72</v>
       </c>
       <c r="J5" t="s">
-        <v>76</v>
+        <v>139</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
         <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D6" t="s">
         <v>62</v>
       </c>
       <c r="E6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F6">
         <v>1.2</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" t="s">
         <v>8</v>
       </c>
       <c r="I6" t="s">
-        <v>72</v>
+        <v>136</v>
       </c>
       <c r="J6" t="s">
-        <v>76</v>
+        <v>140</v>
       </c>
       <c r="K6">
         <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" t="s">
+        <v>134</v>
+      </c>
+      <c r="F7">
+        <v>1.3</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>135</v>
+      </c>
+      <c r="I7" t="s">
+        <v>137</v>
+      </c>
+      <c r="J7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" t="s">
+        <v>143</v>
+      </c>
+      <c r="C8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" t="s">
+        <v>144</v>
+      </c>
+      <c r="F8">
+        <v>1.4</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>135</v>
+      </c>
+      <c r="I8" t="s">
+        <v>145</v>
+      </c>
+      <c r="J8" t="s">
+        <v>146</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1002,7 +1312,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C70B00-7E47-4939-BD03-7BD8F4F3F11B}">
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:R67"/>
   <sheetFormatPr defaultColWidth="18.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" customWidth="1"/>
@@ -1441,7 +1751,7 @@
         <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1467,7 +1777,7 @@
         <v>13</v>
       </c>
       <c r="E18" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -1614,10 +1924,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>63</v>
+        <v>179</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>63</v>
+        <v>179</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>65</v>
@@ -1767,16 +2077,16 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B30" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C30" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>14</v>
@@ -1793,16 +2103,16 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" t="s">
         <v>89</v>
       </c>
-      <c r="B31" t="s">
-        <v>84</v>
-      </c>
-      <c r="C31" t="s">
-        <v>91</v>
-      </c>
       <c r="D31" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>59</v>
@@ -1819,16 +2129,16 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B32" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C32" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>17</v>
@@ -1843,18 +2153,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B33" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C33" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E33" t="s">
         <v>18</v>
@@ -1869,18 +2179,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B34" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C34" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E34" t="s">
         <v>19</v>
@@ -1895,18 +2205,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B35" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C35" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E35" t="s">
         <v>20</v>
@@ -1921,19 +2231,769 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>131</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="H36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>131</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>131</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>94</v>
+      </c>
       <c r="E38" s="6"/>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-      <c r="H38" s="6"/>
-      <c r="I38" s="6"/>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>131</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <v>0</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>131</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>131</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41">
+        <v>0</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>131</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>131</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>131</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>131</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>131</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>0</v>
+      </c>
+      <c r="H46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>131</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
+        <v>0</v>
+      </c>
+      <c r="H47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>131</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48">
+        <v>0</v>
+      </c>
+      <c r="H48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>131</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E49" s="8"/>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49">
+        <v>0</v>
+      </c>
+      <c r="I49" s="8"/>
+      <c r="J49" s="8"/>
+      <c r="K49" s="8"/>
+      <c r="L49" s="8"/>
+      <c r="M49" s="8"/>
+      <c r="N49" s="8"/>
+      <c r="O49" s="8"/>
+      <c r="P49" s="8"/>
+      <c r="Q49" s="8"/>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>131</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+      <c r="G50">
+        <v>0</v>
+      </c>
+      <c r="H50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>131</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+      <c r="G51">
+        <v>0</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>142</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="G52">
+        <v>1</v>
+      </c>
+      <c r="H52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>142</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F53">
+        <v>0</v>
+      </c>
+      <c r="G53">
+        <v>0</v>
+      </c>
+      <c r="H53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>142</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F54">
+        <v>1</v>
+      </c>
+      <c r="G54">
+        <v>0</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>142</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>142</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="G56">
+        <v>0</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>142</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E57" s="9"/>
+      <c r="F57">
+        <v>0</v>
+      </c>
+      <c r="G57">
+        <v>0</v>
+      </c>
+      <c r="H57">
+        <v>0</v>
+      </c>
+      <c r="I57" s="9"/>
+      <c r="J57" s="9"/>
+      <c r="K57" s="9"/>
+      <c r="L57" s="9"/>
+      <c r="M57" s="9"/>
+      <c r="N57" s="9"/>
+      <c r="O57" s="9"/>
+      <c r="P57" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="Q57" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="R57" s="10" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>142</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F58">
+        <v>0</v>
+      </c>
+      <c r="G58">
+        <v>0</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>142</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F59">
+        <v>0</v>
+      </c>
+      <c r="G59">
+        <v>0</v>
+      </c>
+      <c r="H59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>142</v>
+      </c>
+      <c r="B60" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F60">
+        <v>0</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>142</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F61">
+        <v>0</v>
+      </c>
+      <c r="G61">
+        <v>0</v>
+      </c>
+      <c r="H61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>142</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F62">
+        <v>0</v>
+      </c>
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>142</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C63" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F63">
+        <v>0</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>142</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F64">
+        <v>0</v>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>142</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>142</v>
+      </c>
+      <c r="B66" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C66" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F66">
+        <v>0</v>
+      </c>
+      <c r="G66">
+        <v>0</v>
+      </c>
+      <c r="H66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>142</v>
+      </c>
+      <c r="B67" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F67">
+        <v>0</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix DW table generation: correct ordering of SCD2 + common metadata columns (no duplicates)
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC68DB1E-4053-47DC-BF4E-A7D3C141997A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E54F465-7C4C-47CA-905C-861C2E10F2AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
@@ -1295,7 +1295,7 @@
         <v>145</v>
       </c>
       <c r="K8">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Align format file path to config\format folder (consistent with etl_config)
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E54F465-7C4C-47CA-905C-861C2E10F2AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9706A144-0186-4948-9027-C017ABD9925B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
@@ -1190,7 +1190,7 @@
         <v>138</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1295,7 +1295,7 @@
         <v>145</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
testing etl orchestrator 1
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9706A144-0186-4948-9027-C017ABD9925B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39932047-5891-4EF3-914E-5774E2065933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="183">
   <si>
     <t>Source_Name</t>
   </si>
@@ -622,18 +622,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -649,7 +643,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -661,7 +655,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1085,7 +1078,7 @@
         <v>75</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1120,7 +1113,7 @@
         <v>76</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1190,7 +1183,7 @@
         <v>138</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1305,7 +1298,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C70B00-7E47-4939-BD03-7BD8F4F3F11B}">
-  <dimension ref="A1:R67"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr defaultColWidth="18.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" customWidth="1"/>
@@ -1314,29 +1307,29 @@
     <col min="5" max="5" width="44" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8" t="s">
+    <row r="1" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="7" t="s">
         <v>65</v>
       </c>
     </row>
@@ -2524,7 +2517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>130</v>
       </c>
@@ -2547,17 +2540,8 @@
       <c r="H49">
         <v>0</v>
       </c>
-      <c r="I49" s="4"/>
-      <c r="J49" s="4"/>
-      <c r="K49" s="4"/>
-      <c r="L49" s="4"/>
-      <c r="M49" s="4"/>
-      <c r="N49" s="4"/>
-      <c r="O49" s="4"/>
-      <c r="P49" s="4"/>
-      <c r="Q49" s="4"/>
-    </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>130</v>
       </c>
@@ -2580,7 +2564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>130</v>
       </c>
@@ -2603,7 +2587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>141</v>
       </c>
@@ -2626,7 +2610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>141</v>
       </c>
@@ -2652,7 +2636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>141</v>
       </c>
@@ -2678,7 +2662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>141</v>
       </c>
@@ -2704,7 +2688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>141</v>
       </c>
@@ -2730,7 +2714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>141</v>
       </c>
@@ -2755,24 +2739,8 @@
       <c r="H57">
         <v>0</v>
       </c>
-      <c r="I57" s="4"/>
-      <c r="J57" s="4"/>
-      <c r="K57" s="4"/>
-      <c r="L57" s="4"/>
-      <c r="M57" s="4"/>
-      <c r="N57" s="4"/>
-      <c r="O57" s="4"/>
-      <c r="P57" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q57" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="R57" s="7" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>141</v>
       </c>
@@ -2798,7 +2766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>141</v>
       </c>
@@ -2824,7 +2792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>141</v>
       </c>
@@ -2850,7 +2818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>141</v>
       </c>
@@ -2873,7 +2841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>141</v>
       </c>
@@ -2896,7 +2864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>141</v>
       </c>
@@ -2919,7 +2887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>141</v>
       </c>

</xml_diff>

<commit_message>
updated ETL Files and tables
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SISRI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F3DA6D-E11A-4365-8FDD-01B95A9DC24E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA9FBD5-29E7-4A6E-A760-E389A3F08036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
     <sheet name="Source_File_Mapping" sheetId="2" r:id="rId2"/>
-    <sheet name="Fact_Conformed_Mapping" sheetId="3" r:id="rId3"/>
+    <sheet name="DW_Mapping_And_Transformations" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="260">
   <si>
     <t>Source_Name</t>
   </si>
@@ -700,117 +700,131 @@
     <t>DateLookup</t>
   </si>
   <si>
-    <t>EOMONTH(PARSE_DATE(ODS_Column, 'dd-MM-yyyy')) → lookup Dim_Date</t>
-  </si>
-  <si>
-    <t>Required</t>
-  </si>
-  <si>
     <t>ExtractCode</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">REGEX '\d+ \d+ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFCC0000"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>\d</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>+' from ODS_Column</t>
-    </r>
-  </si>
-  <si>
-    <t>First part before space or specific prefix</t>
-  </si>
-  <si>
     <t>Direct</t>
   </si>
   <si>
-    <t>DIRECT</t>
-  </si>
-  <si>
     <t>Convert</t>
   </si>
   <si>
-    <t>CAST AS DECIMAL(18,4)</t>
-  </si>
-  <si>
-    <t>&gt;0 or allow neg</t>
-  </si>
-  <si>
     <t>Total_Amount_Source</t>
   </si>
   <si>
-    <t>CAST AS DECIMAL(18,4), strip 'R'</t>
-  </si>
-  <si>
     <t>Unit_Cost_Price</t>
   </si>
   <si>
     <t>NULL</t>
   </si>
   <si>
-    <t>All</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Unit_Price</t>
-  </si>
-  <si>
-    <t>Calculated</t>
-  </si>
-  <si>
-    <t>NULL for now (or map from another column later)</t>
-  </si>
-  <si>
-    <t>Total_Amount_Calc</t>
-  </si>
-  <si>
-    <t>Sales_Quantity * ISNULL(Unit_Price, Unit_Cost_Price)</t>
-  </si>
-  <si>
-    <t>Match source ±0.01</t>
-  </si>
-  <si>
-    <t>Fact_Conformed_Mapping</t>
-  </si>
-  <si>
-    <t>[ETL].[Fact_Conformed_Mapping]</t>
-  </si>
-  <si>
     <t>Fact key fields mapping</t>
   </si>
   <si>
-    <t>[ETL].[Dim_Fact_Conformed_Mapping]</t>
-  </si>
-  <si>
-    <t>[ETL].[[SP_Merge_Dim_Fact_Conformed_Mapping]</t>
-  </si>
-  <si>
     <t>VARCHAR(2000)</t>
+  </si>
+  <si>
+    <t>DW_Mapping_And_Transformations</t>
+  </si>
+  <si>
+    <t>[ETL].[Dim_DW_Mapping_And_Transformations]</t>
+  </si>
+  <si>
+    <t>[ETL].[[SP_Merge_Dim_DW_Mapping_And_Transformations]</t>
+  </si>
+  <si>
+    <t>[ETL].[DW_Mapping_And_Transformations]</t>
+  </si>
+  <si>
+    <t>UNKNOWN</t>
+  </si>
+  <si>
+    <t>[ETL].[Staging_Fact_Sales_Conformed]</t>
+  </si>
+  <si>
+    <t>[ETL].[SP_Merge_Sales_Format_1_To_Staging_Fact_Sales_Conformed]</t>
+  </si>
+  <si>
+    <t>SourceFileName</t>
+  </si>
+  <si>
+    <t>TRY_CAST(REPLACE(ODS_Column, ',', ') AS DECIMAL(18,4))</t>
+  </si>
+  <si>
+    <t>LTRIM(RTRIM(LEFT(ODS_Column, CHARINDEX(' ', ODS_Column + ' ') - 1)))</t>
+  </si>
+  <si>
+    <t>TRY_CAST(REPLACE(REPLACE(ODS_Column, 'R', ''), ',', ') AS DECIMAL(18,4))</t>
+  </si>
+  <si>
+    <t>CONVERT(INT, CONVERT(VARCHAR(8), EOMONTH(TRY_PARSE(REPLACE(ODS_Column, '/', '-') AS DATE USING 'en-ZA')), 112))</t>
+  </si>
+  <si>
+    <t>LTRIM(RTRIM(SUBSTRING(ODS_Column, CHARINDEX('(', ODS_Column) + 1, CHARINDEX(')', ODS_Column) - CHARINDEX('(', ODS_Column) - 1)))</t>
+  </si>
+  <si>
+    <t>Direct pass-through, default UNKNOWN if NULL/empty</t>
+  </si>
+  <si>
+    <t>Clean commas ? DECIMAL(18,4)</t>
+  </si>
+  <si>
+    <t>Required - first word/prefix</t>
+  </si>
+  <si>
+    <t>Take left part up to first space e.g. CL377862 WEDGEWOOD ANGEL BISCUIT ? CL377862</t>
+  </si>
+  <si>
+    <t>Required - numeric amount</t>
+  </si>
+  <si>
+    <t>Remove R + commas ? DECIMAL(18,4)</t>
+  </si>
+  <si>
+    <t>Valid date required</t>
+  </si>
+  <si>
+    <t>Convert dd-MM-yyyy or dd/MM/yyyy ? last day of month ? yyyyMMdd integer (Dim_Date key)</t>
+  </si>
+  <si>
+    <t>Numeric, allow negative for returns</t>
+  </si>
+  <si>
+    <t>Required - audit field</t>
+  </si>
+  <si>
+    <t>Direct pass-through from ODS</t>
+  </si>
+  <si>
+    <t>Required - code in parentheses</t>
+  </si>
+  <si>
+    <t>Extract numeric code inside parentheses e.g. (1931) ? 1931</t>
+  </si>
+  <si>
+    <t>Sequence_Order</t>
+  </si>
+  <si>
+    <t>Is_Conformed_Target</t>
+  </si>
+  <si>
+    <t>Staging_Fact_Sales_Conformed</t>
+  </si>
+  <si>
+    <t>Conformed staging target for all Fact_Sales sources</t>
+  </si>
+  <si>
+    <t>Fact_Conformed</t>
+  </si>
+  <si>
+    <t>Indicates if multiple sources are conformed into a single table</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -845,13 +859,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFCC0000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -874,7 +881,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -900,6 +907,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1236,23 +1249,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{584572B9-381C-487F-864D-5B674FBBA046}">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="45" customWidth="1"/>
+    <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.28515625" customWidth="1"/>
-    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
     <col min="8" max="8" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="32.140625" customWidth="1"/>
-    <col min="10" max="10" width="43.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="43.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.5703125" customWidth="1"/>
+    <col min="13" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1289,8 +1303,11 @@
       <c r="L1" s="1" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -1327,8 +1344,11 @@
       <c r="L2" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1365,10 +1385,13 @@
       <c r="L3" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="B4" t="s">
         <v>25</v>
@@ -1377,10 +1400,10 @@
         <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E4" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="F4">
         <v>0.12</v>
@@ -1389,13 +1412,13 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>244</v>
+        <v>226</v>
       </c>
       <c r="I4" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="J4" t="s">
-        <v>246</v>
+        <v>230</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -1403,8 +1426,11 @@
       <c r="L4" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1441,8 +1467,11 @@
       <c r="L5" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1479,8 +1508,11 @@
       <c r="L6" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>86</v>
       </c>
@@ -1517,8 +1549,11 @@
       <c r="L7" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>130</v>
       </c>
@@ -1555,8 +1590,11 @@
       <c r="L8" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>141</v>
       </c>
@@ -1593,8 +1631,11 @@
       <c r="L9" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>183</v>
       </c>
@@ -1620,16 +1661,60 @@
         <v>186</v>
       </c>
       <c r="I10" t="s">
-        <v>187</v>
+        <v>233</v>
       </c>
       <c r="J10" t="s">
-        <v>188</v>
+        <v>234</v>
       </c>
       <c r="K10">
         <v>1</v>
       </c>
       <c r="L10" t="s">
         <v>204</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>256</v>
+      </c>
+      <c r="B11" t="s">
+        <v>225</v>
+      </c>
+      <c r="C11" t="s">
+        <v>225</v>
+      </c>
+      <c r="D11" t="s">
+        <v>225</v>
+      </c>
+      <c r="E11" t="s">
+        <v>233</v>
+      </c>
+      <c r="F11">
+        <v>3.01</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>257</v>
+      </c>
+      <c r="I11" t="s">
+        <v>187</v>
+      </c>
+      <c r="J11" t="s">
+        <v>188</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11" t="s">
+        <v>258</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1639,7 +1724,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C70B00-7E47-4939-BD03-7BD8F4F3F11B}">
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr defaultColWidth="18.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" customWidth="1"/>
@@ -2144,25 +2229,25 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="B20" t="s">
+        <v>255</v>
+      </c>
+      <c r="C20" t="s">
+        <v>255</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>205</v>
+        <v>64</v>
       </c>
       <c r="E20" t="s">
-        <v>40</v>
+        <v>259</v>
       </c>
       <c r="F20">
         <v>0</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -2173,16 +2258,16 @@
         <v>23</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>13</v>
+        <v>205</v>
       </c>
       <c r="E21" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -2199,22 +2284,22 @@
         <v>23</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E22" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -2225,16 +2310,16 @@
         <v>23</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -2251,16 +2336,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -2269,7 +2354,7 @@
         <v>0</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -2277,16 +2362,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>178</v>
+        <v>6</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>178</v>
+        <v>6</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E25" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -2295,7 +2380,7 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -2303,16 +2388,16 @@
         <v>23</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>63</v>
+        <v>178</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>63</v>
+        <v>178</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>64</v>
       </c>
       <c r="E26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -2329,16 +2414,16 @@
         <v>23</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>64</v>
       </c>
       <c r="E27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -2352,25 +2437,25 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>9</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>29</v>
+        <v>23</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>14</v>
+        <v>64</v>
+      </c>
+      <c r="E28" t="s">
+        <v>68</v>
       </c>
       <c r="F28">
         <v>0</v>
       </c>
       <c r="G28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H28">
         <v>1</v>
@@ -2381,10 +2466,10 @@
         <v>9</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>57</v>
+        <v>48</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>13</v>
@@ -2407,22 +2492,22 @@
         <v>9</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E30" t="s">
-        <v>59</v>
+      <c r="E30" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="F30">
         <v>0</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H30">
         <v>1</v>
@@ -2430,25 +2515,25 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>86</v>
-      </c>
-      <c r="B31" t="s">
-        <v>80</v>
-      </c>
-      <c r="C31" t="s">
-        <v>87</v>
+        <v>9</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>58</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="E31" t="s">
+        <v>59</v>
       </c>
       <c r="F31">
         <v>0</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H31">
         <v>1</v>
@@ -2459,22 +2544,22 @@
         <v>86</v>
       </c>
       <c r="B32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C32" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="F32">
         <v>0</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H32">
         <v>1</v>
@@ -2485,16 +2570,16 @@
         <v>86</v>
       </c>
       <c r="B33" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C33" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="F33">
         <v>0</v>
@@ -2503,7 +2588,7 @@
         <v>0</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -2511,16 +2596,16 @@
         <v>86</v>
       </c>
       <c r="B34" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C34" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E34" t="s">
-        <v>18</v>
+      <c r="E34" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -2537,16 +2622,16 @@
         <v>86</v>
       </c>
       <c r="B35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C35" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F35">
         <v>0</v>
@@ -2563,16 +2648,16 @@
         <v>86</v>
       </c>
       <c r="B36" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C36" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F36">
         <v>0</v>
@@ -2586,25 +2671,28 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>130</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>116</v>
+        <v>86</v>
+      </c>
+      <c r="B37" t="s">
+        <v>85</v>
+      </c>
+      <c r="C37" t="s">
+        <v>92</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="E37" t="s">
+        <v>20</v>
+      </c>
       <c r="F37">
         <v>0</v>
       </c>
       <c r="G37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H37">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -2612,10 +2700,10 @@
         <v>130</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>93</v>
@@ -2624,7 +2712,7 @@
         <v>0</v>
       </c>
       <c r="G38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H38">
         <v>1</v>
@@ -2635,15 +2723,14 @@
         <v>130</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E39" s="5"/>
       <c r="F39">
         <v>0</v>
       </c>
@@ -2659,14 +2746,15 @@
         <v>130</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>29</v>
+        <v>102</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>118</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="E40" s="5"/>
       <c r="F40">
         <v>0</v>
       </c>
@@ -2682,10 +2770,10 @@
         <v>130</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>57</v>
+        <v>103</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>93</v>
@@ -2705,10 +2793,10 @@
         <v>130</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>119</v>
+        <v>57</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>93</v>
@@ -2720,7 +2808,7 @@
         <v>0</v>
       </c>
       <c r="H42">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -2728,10 +2816,10 @@
         <v>130</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>93</v>
@@ -2751,10 +2839,10 @@
         <v>130</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>93</v>
@@ -2774,10 +2862,10 @@
         <v>130</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>93</v>
@@ -2797,10 +2885,10 @@
         <v>130</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>93</v>
@@ -2820,10 +2908,10 @@
         <v>130</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>93</v>
@@ -2843,10 +2931,10 @@
         <v>130</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>93</v>
@@ -2866,10 +2954,10 @@
         <v>130</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>93</v>
@@ -2889,15 +2977,14 @@
         <v>130</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E50" s="4"/>
       <c r="F50">
         <v>0</v>
       </c>
@@ -2913,14 +3000,15 @@
         <v>130</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="E51" s="4"/>
       <c r="F51">
         <v>0</v>
       </c>
@@ -2936,10 +3024,10 @@
         <v>130</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>93</v>
@@ -2956,13 +3044,13 @@
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>146</v>
+        <v>115</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>162</v>
+        <v>129</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>93</v>
@@ -2971,10 +3059,10 @@
         <v>0</v>
       </c>
       <c r="G53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H53">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
@@ -2982,22 +3070,19 @@
         <v>141</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E54" t="s">
-        <v>59</v>
-      </c>
       <c r="F54">
         <v>0</v>
       </c>
       <c r="G54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H54">
         <v>1</v>
@@ -3008,25 +3093,25 @@
         <v>141</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E55" t="s">
-        <v>179</v>
+        <v>59</v>
       </c>
       <c r="F55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G55">
         <v>0</v>
       </c>
       <c r="H55">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -3034,16 +3119,16 @@
         <v>141</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E56" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F56">
         <v>1</v>
@@ -3060,19 +3145,19 @@
         <v>141</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E57" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F57">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G57">
         <v>0</v>
@@ -3086,16 +3171,16 @@
         <v>141</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E58" s="4" t="s">
-        <v>181</v>
+      <c r="E58" t="s">
+        <v>180</v>
       </c>
       <c r="F58">
         <v>0</v>
@@ -3112,16 +3197,16 @@
         <v>141</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E59" t="s">
-        <v>18</v>
+      <c r="E59" s="4" t="s">
+        <v>181</v>
       </c>
       <c r="F59">
         <v>0</v>
@@ -3138,16 +3223,16 @@
         <v>141</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E60" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F60">
         <v>0</v>
@@ -3164,16 +3249,16 @@
         <v>141</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E61" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F61">
         <v>0</v>
@@ -3190,13 +3275,16 @@
         <v>141</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>93</v>
+      </c>
+      <c r="E62" t="s">
+        <v>20</v>
       </c>
       <c r="F62">
         <v>0</v>
@@ -3213,10 +3301,10 @@
         <v>141</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>93</v>
@@ -3236,10 +3324,10 @@
         <v>141</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>93</v>
@@ -3259,10 +3347,10 @@
         <v>141</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>93</v>
@@ -3282,10 +3370,10 @@
         <v>141</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>93</v>
@@ -3305,10 +3393,10 @@
         <v>141</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>93</v>
@@ -3328,10 +3416,10 @@
         <v>141</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>93</v>
@@ -3348,28 +3436,25 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>183</v>
+        <v>141</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>189</v>
+        <v>161</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E69" s="4" t="s">
-        <v>189</v>
-      </c>
       <c r="F69">
         <v>0</v>
       </c>
       <c r="G69">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H69">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -3377,16 +3462,16 @@
         <v>183</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>101</v>
+        <v>189</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>117</v>
+        <v>194</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>101</v>
+        <v>189</v>
       </c>
       <c r="F70">
         <v>0</v>
@@ -3403,16 +3488,16 @@
         <v>183</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>190</v>
+        <v>101</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>195</v>
+        <v>117</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E71" t="s">
-        <v>210</v>
+      <c r="E71" s="4" t="s">
+        <v>101</v>
       </c>
       <c r="F71">
         <v>0</v>
@@ -3429,19 +3514,22 @@
         <v>183</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="E72" t="s">
+        <v>210</v>
+      </c>
       <c r="F72">
         <v>0</v>
       </c>
       <c r="G72">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H72">
         <v>1</v>
@@ -3452,13 +3540,13 @@
         <v>183</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="D73" t="s">
-        <v>196</v>
+        <v>191</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="F73">
         <v>0</v>
@@ -3475,13 +3563,13 @@
         <v>183</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
+      </c>
+      <c r="D74" t="s">
+        <v>196</v>
       </c>
       <c r="F74">
         <v>0</v>
@@ -3497,14 +3585,14 @@
       <c r="A75" t="s">
         <v>183</v>
       </c>
-      <c r="B75" t="s">
-        <v>209</v>
+      <c r="B75" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="D75" t="s">
-        <v>196</v>
+        <v>199</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>197</v>
       </c>
       <c r="F75">
         <v>0</v>
@@ -3518,22 +3606,22 @@
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>242</v>
-      </c>
-      <c r="B76" s="4" t="s">
-        <v>0</v>
+        <v>183</v>
+      </c>
+      <c r="B76" t="s">
+        <v>209</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>93</v>
+        <v>200</v>
+      </c>
+      <c r="D76" t="s">
+        <v>196</v>
       </c>
       <c r="F76">
         <v>0</v>
       </c>
       <c r="G76">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H76">
         <v>1</v>
@@ -3541,13 +3629,13 @@
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>93</v>
@@ -3564,23 +3652,22 @@
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E78" s="9"/>
       <c r="F78">
         <v>0</v>
       </c>
       <c r="G78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H78">
         <v>1</v>
@@ -3588,17 +3675,18 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="E79" s="9"/>
       <c r="F79">
         <v>0</v>
       </c>
@@ -3611,13 +3699,13 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>93</v>
@@ -3629,21 +3717,21 @@
         <v>0</v>
       </c>
       <c r="H80">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="F81">
         <v>0</v>
@@ -3657,13 +3745,13 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>65</v>
+        <v>215</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>65</v>
+        <v>215</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>64</v>
@@ -3680,16 +3768,16 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>216</v>
+        <v>65</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>216</v>
+        <v>65</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="F83">
         <v>0</v>
@@ -3703,29 +3791,95 @@
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="B84" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F84">
+        <v>0</v>
+      </c>
+      <c r="G84">
+        <v>0</v>
+      </c>
+      <c r="H84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>228</v>
+      </c>
+      <c r="B85" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="C84" s="4" t="s">
+      <c r="C85" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="D84" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F84">
-        <v>0</v>
-      </c>
-      <c r="G84">
-        <v>0</v>
-      </c>
-      <c r="H84">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D85" s="2"/>
+      <c r="D85" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="F85">
+        <v>0</v>
+      </c>
+      <c r="G85">
+        <v>0</v>
+      </c>
+      <c r="H85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>228</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F86">
+        <v>0</v>
+      </c>
+      <c r="G86">
+        <v>0</v>
+      </c>
+      <c r="H86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>228</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F87">
+        <v>0</v>
+      </c>
+      <c r="G87">
+        <v>0</v>
+      </c>
+      <c r="H87">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -3736,7 +3890,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0143FCE7-ABA4-4505-A711-BECADC2D92A0}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultColWidth="65.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.85546875" style="10" bestFit="1" customWidth="1"/>
@@ -3748,10 +3902,11 @@
     <col min="7" max="7" width="11.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="65.7109375" style="10"/>
+    <col min="10" max="10" width="18.140625" style="10" customWidth="1"/>
+    <col min="11" max="16384" width="65.7109375" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -3779,76 +3934,98 @@
       <c r="I1" s="9" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J1" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="K1" s="13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>183</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>218</v>
+        <v>191</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="F2" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="11">
-        <v>1</v>
-      </c>
-      <c r="H2" s="11"/>
+        <v>0</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>232</v>
+      </c>
       <c r="I2" s="11" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>225</v>
+      </c>
+      <c r="J2" s="11">
+        <v>4</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>183</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>189</v>
+        <v>209</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>162</v>
+        <v>224</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>222</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="F3" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" s="11">
-        <v>1</v>
-      </c>
-      <c r="H3" s="11"/>
+        <v>0</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>225</v>
+      </c>
       <c r="I3" s="11" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>225</v>
+      </c>
+      <c r="J3" s="11">
+        <v>6</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>183</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>116</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="F4" s="11">
         <v>1</v>
@@ -3856,80 +4033,104 @@
       <c r="G4" s="11">
         <v>1</v>
       </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="11" t="s">
+        <v>232</v>
+      </c>
       <c r="I4" s="11" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>243</v>
+      </c>
+      <c r="J4" s="11">
+        <v>3</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>183</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>191</v>
+        <v>223</v>
       </c>
       <c r="D5" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="F5" s="11">
+        <v>0</v>
+      </c>
+      <c r="G5" s="11">
+        <v>1</v>
+      </c>
+      <c r="H5" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="E5" s="11" t="s">
-        <v>226</v>
-      </c>
-      <c r="F5" s="11">
-        <v>0</v>
-      </c>
-      <c r="G5" s="11">
-        <v>0</v>
-      </c>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I5" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="J5" s="11">
+        <v>7</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>183</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="F6" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="11">
         <v>1</v>
       </c>
       <c r="H6" s="11">
-        <v>0</v>
+        <v>19000101</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>247</v>
+      </c>
+      <c r="J6" s="11">
+        <v>1</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>183</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>230</v>
+        <v>199</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="F7" s="11">
         <v>0</v>
@@ -3937,93 +4138,91 @@
       <c r="G7" s="11">
         <v>1</v>
       </c>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H7" s="11">
+        <v>0</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J7" s="11">
+        <v>5</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>183</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>209</v>
+        <v>235</v>
       </c>
       <c r="C8" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="F8" s="11">
+        <v>0</v>
+      </c>
+      <c r="G8" s="11">
+        <v>1</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="J8" s="11">
+        <v>8</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="F9" s="11">
+        <v>1</v>
+      </c>
+      <c r="G9" s="11">
+        <v>1</v>
+      </c>
+      <c r="H9" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="D8" s="11" t="s">
-        <v>227</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="F8" s="11">
-        <v>0</v>
-      </c>
-      <c r="G8" s="11">
-        <v>0</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="I8" s="11"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>234</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>235</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>237</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>238</v>
-      </c>
-      <c r="F9" s="11">
-        <v>0</v>
-      </c>
-      <c r="G9" s="11">
-        <v>0</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="I9" s="11"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>234</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>235</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>239</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>237</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>240</v>
-      </c>
-      <c r="F10" s="11">
-        <v>0</v>
-      </c>
-      <c r="G10" s="11">
-        <v>0</v>
-      </c>
-      <c r="H10" s="11">
-        <v>0</v>
-      </c>
-      <c r="I10" s="11" t="s">
-        <v>241</v>
+      <c r="I9" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="J9" s="11">
+        <v>2</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>253</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
More conformed fact stuff
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SISRI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA9FBD5-29E7-4A6E-A760-E389A3F08036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC5D2F3-9C6A-432A-B3ED-0F7F9659C58E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{E5D07F8F-8FAA-4189-8D8F-833E9D798696}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="257">
   <si>
     <t>Source_Name</t>
   </si>
@@ -697,18 +697,9 @@
     <t>Date_SK</t>
   </si>
   <si>
-    <t>DateLookup</t>
-  </si>
-  <si>
-    <t>ExtractCode</t>
-  </si>
-  <si>
     <t>Direct</t>
   </si>
   <si>
-    <t>Convert</t>
-  </si>
-  <si>
     <t>Total_Amount_Source</t>
   </si>
   <si>
@@ -736,33 +727,12 @@
     <t>[ETL].[DW_Mapping_And_Transformations]</t>
   </si>
   <si>
-    <t>UNKNOWN</t>
-  </si>
-  <si>
     <t>[ETL].[Staging_Fact_Sales_Conformed]</t>
   </si>
   <si>
     <t>[ETL].[SP_Merge_Sales_Format_1_To_Staging_Fact_Sales_Conformed]</t>
   </si>
   <si>
-    <t>SourceFileName</t>
-  </si>
-  <si>
-    <t>TRY_CAST(REPLACE(ODS_Column, ',', ') AS DECIMAL(18,4))</t>
-  </si>
-  <si>
-    <t>LTRIM(RTRIM(LEFT(ODS_Column, CHARINDEX(' ', ODS_Column + ' ') - 1)))</t>
-  </si>
-  <si>
-    <t>TRY_CAST(REPLACE(REPLACE(ODS_Column, 'R', ''), ',', ') AS DECIMAL(18,4))</t>
-  </si>
-  <si>
-    <t>CONVERT(INT, CONVERT(VARCHAR(8), EOMONTH(TRY_PARSE(REPLACE(ODS_Column, '/', '-') AS DATE USING 'en-ZA')), 112))</t>
-  </si>
-  <si>
-    <t>LTRIM(RTRIM(SUBSTRING(ODS_Column, CHARINDEX('(', ODS_Column) + 1, CHARINDEX(')', ODS_Column) - CHARINDEX('(', ODS_Column) - 1)))</t>
-  </si>
-  <si>
     <t>Direct pass-through, default UNKNOWN if NULL/empty</t>
   </si>
   <si>
@@ -790,12 +760,6 @@
     <t>Numeric, allow negative for returns</t>
   </si>
   <si>
-    <t>Required - audit field</t>
-  </si>
-  <si>
-    <t>Direct pass-through from ODS</t>
-  </si>
-  <si>
     <t>Required - code in parentheses</t>
   </si>
   <si>
@@ -818,6 +782,33 @@
   </si>
   <si>
     <t>Indicates if multiple sources are conformed into a single table</t>
+  </si>
+  <si>
+    <t>Expression</t>
+  </si>
+  <si>
+    <t>'UNKNOWN'</t>
+  </si>
+  <si>
+    <t>[Sales_Amount]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CONVERT(INT, CONVERT(VARCHAR(8), TRY_CONVERT(DATE,[Sales_Date_dd-MM-YYYY], 105), 112))</t>
+  </si>
+  <si>
+    <t>[Sales_Quantity]</t>
+  </si>
+  <si>
+    <t>[Store_Name]</t>
+  </si>
+  <si>
+    <t>[Barcode]</t>
+  </si>
+  <si>
+    <t>LEFT([Product_Name], CHARINDEX(' ', [Product_Name] + ' ') - 1)</t>
+  </si>
+  <si>
+    <t>[Cost_Price]</t>
   </si>
 </sst>
 </file>
@@ -881,7 +872,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -908,12 +899,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1249,7 +1244,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{584572B9-381C-487F-864D-5B674FBBA046}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
@@ -1263,10 +1258,11 @@
     <col min="9" max="10" width="43.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.5703125" customWidth="1"/>
     <col min="13" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1304,10 +1300,13 @@
         <v>201</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+        <v>243</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -1348,7 +1347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1389,9 +1388,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B4" t="s">
         <v>25</v>
@@ -1400,10 +1399,10 @@
         <v>26</v>
       </c>
       <c r="D4" t="s">
+        <v>225</v>
+      </c>
+      <c r="E4" t="s">
         <v>228</v>
-      </c>
-      <c r="E4" t="s">
-        <v>231</v>
       </c>
       <c r="F4">
         <v>0.12</v>
@@ -1412,13 +1411,13 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
+        <v>223</v>
+      </c>
+      <c r="I4" t="s">
         <v>226</v>
       </c>
-      <c r="I4" t="s">
-        <v>229</v>
-      </c>
       <c r="J4" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -1430,7 +1429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1471,7 +1470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1512,7 +1511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>86</v>
       </c>
@@ -1553,7 +1552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>130</v>
       </c>
@@ -1594,7 +1593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>141</v>
       </c>
@@ -1635,7 +1634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>183</v>
       </c>
@@ -1661,10 +1660,10 @@
         <v>186</v>
       </c>
       <c r="I10" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="J10" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="K10">
         <v>1</v>
@@ -1676,21 +1675,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="B11" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C11" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D11" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E11" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="F11">
         <v>3.01</v>
@@ -1699,7 +1698,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="I11" t="s">
         <v>187</v>
@@ -1711,7 +1710,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="M11">
         <v>0</v>
@@ -1724,7 +1723,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C70B00-7E47-4939-BD03-7BD8F4F3F11B}">
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr defaultColWidth="18.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" customWidth="1"/>
@@ -1770,7 +1769,7 @@
         <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>14</v>
@@ -1796,7 +1795,7 @@
         <v>30</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>15</v>
@@ -1822,7 +1821,7 @@
         <v>31</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>16</v>
@@ -1848,7 +1847,7 @@
         <v>32</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>17</v>
@@ -1874,7 +1873,7 @@
         <v>33</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E6" t="s">
         <v>18</v>
@@ -1900,7 +1899,7 @@
         <v>34</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E7" t="s">
         <v>19</v>
@@ -1926,7 +1925,7 @@
         <v>35</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E8" t="s">
         <v>20</v>
@@ -2232,16 +2231,16 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="C20" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>64</v>
       </c>
       <c r="E20" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -2255,28 +2254,28 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="E21" t="s">
-        <v>40</v>
+        <v>93</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>80</v>
       </c>
       <c r="F21">
         <v>0</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -2284,16 +2283,16 @@
         <v>23</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>13</v>
+        <v>205</v>
       </c>
       <c r="E22" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -2310,22 +2309,22 @@
         <v>23</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E23" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F23">
         <v>0</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23">
         <v>1</v>
@@ -2336,16 +2335,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -2362,16 +2361,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E25" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -2380,7 +2379,7 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -2388,16 +2387,16 @@
         <v>23</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>178</v>
+        <v>6</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>178</v>
+        <v>6</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E26" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -2406,7 +2405,7 @@
         <v>0</v>
       </c>
       <c r="H26">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -2414,16 +2413,16 @@
         <v>23</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>63</v>
+        <v>178</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>63</v>
+        <v>178</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>64</v>
       </c>
       <c r="E27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -2440,16 +2439,16 @@
         <v>23</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>64</v>
       </c>
       <c r="E28" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F28">
         <v>0</v>
@@ -2463,25 +2462,25 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>9</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>29</v>
+        <v>23</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>14</v>
+        <v>64</v>
+      </c>
+      <c r="E29" t="s">
+        <v>68</v>
       </c>
       <c r="F29">
         <v>0</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29">
         <v>1</v>
@@ -2492,13 +2491,13 @@
         <v>9</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>57</v>
+        <v>48</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>14</v>
@@ -2518,22 +2517,22 @@
         <v>9</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E31" t="s">
-        <v>59</v>
+        <v>93</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="F31">
         <v>0</v>
       </c>
       <c r="G31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H31">
         <v>1</v>
@@ -2541,25 +2540,25 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>86</v>
-      </c>
-      <c r="B32" t="s">
-        <v>80</v>
-      </c>
-      <c r="C32" t="s">
-        <v>87</v>
+        <v>9</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>58</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>14</v>
+      <c r="E32" t="s">
+        <v>59</v>
       </c>
       <c r="F32">
         <v>0</v>
       </c>
       <c r="G32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H32">
         <v>1</v>
@@ -2570,22 +2569,22 @@
         <v>86</v>
       </c>
       <c r="B33" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C33" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="F33">
         <v>0</v>
       </c>
       <c r="G33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H33">
         <v>1</v>
@@ -2596,16 +2595,16 @@
         <v>86</v>
       </c>
       <c r="B34" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C34" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -2614,7 +2613,7 @@
         <v>0</v>
       </c>
       <c r="H34">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -2622,16 +2621,16 @@
         <v>86</v>
       </c>
       <c r="B35" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C35" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E35" t="s">
-        <v>18</v>
+      <c r="E35" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="F35">
         <v>0</v>
@@ -2648,16 +2647,16 @@
         <v>86</v>
       </c>
       <c r="B36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F36">
         <v>0</v>
@@ -2674,16 +2673,16 @@
         <v>86</v>
       </c>
       <c r="B37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E37" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F37">
         <v>0</v>
@@ -2697,25 +2696,28 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>130</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>116</v>
+        <v>86</v>
+      </c>
+      <c r="B38" t="s">
+        <v>85</v>
+      </c>
+      <c r="C38" t="s">
+        <v>92</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="E38" t="s">
+        <v>20</v>
+      </c>
       <c r="F38">
         <v>0</v>
       </c>
       <c r="G38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H38">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -2723,10 +2725,10 @@
         <v>130</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>93</v>
@@ -2735,7 +2737,7 @@
         <v>0</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39">
         <v>1</v>
@@ -2746,15 +2748,14 @@
         <v>130</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E40" s="5"/>
       <c r="F40">
         <v>0</v>
       </c>
@@ -2770,14 +2771,15 @@
         <v>130</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>29</v>
+        <v>102</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>118</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="E41" s="5"/>
       <c r="F41">
         <v>0</v>
       </c>
@@ -2793,10 +2795,10 @@
         <v>130</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>57</v>
+        <v>103</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>93</v>
@@ -2816,10 +2818,10 @@
         <v>130</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>119</v>
+        <v>57</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>93</v>
@@ -2831,7 +2833,7 @@
         <v>0</v>
       </c>
       <c r="H43">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -2839,10 +2841,10 @@
         <v>130</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>93</v>
@@ -2862,10 +2864,10 @@
         <v>130</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>93</v>
@@ -2885,10 +2887,10 @@
         <v>130</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>93</v>
@@ -2908,10 +2910,10 @@
         <v>130</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>93</v>
@@ -2931,10 +2933,10 @@
         <v>130</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>93</v>
@@ -2954,10 +2956,10 @@
         <v>130</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>93</v>
@@ -2977,10 +2979,10 @@
         <v>130</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>93</v>
@@ -3000,15 +3002,14 @@
         <v>130</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E51" s="4"/>
       <c r="F51">
         <v>0</v>
       </c>
@@ -3024,14 +3025,15 @@
         <v>130</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="E52" s="4"/>
       <c r="F52">
         <v>0</v>
       </c>
@@ -3047,10 +3049,10 @@
         <v>130</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>93</v>
@@ -3067,13 +3069,13 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>146</v>
+        <v>115</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>162</v>
+        <v>129</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>93</v>
@@ -3082,10 +3084,10 @@
         <v>0</v>
       </c>
       <c r="G54">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H54">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -3093,22 +3095,19 @@
         <v>141</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E55" t="s">
-        <v>59</v>
-      </c>
       <c r="F55">
         <v>0</v>
       </c>
       <c r="G55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H55">
         <v>1</v>
@@ -3119,25 +3118,25 @@
         <v>141</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E56" t="s">
-        <v>179</v>
+        <v>59</v>
       </c>
       <c r="F56">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G56">
         <v>0</v>
       </c>
       <c r="H56">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -3145,16 +3144,16 @@
         <v>141</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E57" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -3171,19 +3170,19 @@
         <v>141</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E58" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G58">
         <v>0</v>
@@ -3197,16 +3196,16 @@
         <v>141</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E59" s="4" t="s">
-        <v>181</v>
+      <c r="E59" t="s">
+        <v>180</v>
       </c>
       <c r="F59">
         <v>0</v>
@@ -3223,16 +3222,16 @@
         <v>141</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E60" t="s">
-        <v>18</v>
+      <c r="E60" s="4" t="s">
+        <v>181</v>
       </c>
       <c r="F60">
         <v>0</v>
@@ -3249,16 +3248,16 @@
         <v>141</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E61" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F61">
         <v>0</v>
@@ -3275,16 +3274,16 @@
         <v>141</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E62" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F62">
         <v>0</v>
@@ -3301,13 +3300,16 @@
         <v>141</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>93</v>
+      </c>
+      <c r="E63" t="s">
+        <v>20</v>
       </c>
       <c r="F63">
         <v>0</v>
@@ -3324,10 +3326,10 @@
         <v>141</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>93</v>
@@ -3347,10 +3349,10 @@
         <v>141</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>93</v>
@@ -3370,10 +3372,10 @@
         <v>141</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>93</v>
@@ -3393,10 +3395,10 @@
         <v>141</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>93</v>
@@ -3416,10 +3418,10 @@
         <v>141</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>93</v>
@@ -3439,10 +3441,10 @@
         <v>141</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>93</v>
@@ -3459,28 +3461,25 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>183</v>
+        <v>141</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>189</v>
+        <v>161</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E70" s="4" t="s">
-        <v>189</v>
-      </c>
       <c r="F70">
         <v>0</v>
       </c>
       <c r="G70">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H70">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
@@ -3488,16 +3487,16 @@
         <v>183</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>101</v>
+        <v>189</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>117</v>
+        <v>194</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>93</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>101</v>
+        <v>189</v>
       </c>
       <c r="F71">
         <v>0</v>
@@ -3514,22 +3513,22 @@
         <v>183</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>190</v>
+        <v>101</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>195</v>
+        <v>117</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E72" t="s">
-        <v>210</v>
+      <c r="E72" s="4" t="s">
+        <v>101</v>
       </c>
       <c r="F72">
         <v>0</v>
       </c>
       <c r="G72">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H72">
         <v>1</v>
@@ -3540,19 +3539,22 @@
         <v>183</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="E73" t="s">
+        <v>210</v>
+      </c>
       <c r="F73">
         <v>0</v>
       </c>
       <c r="G73">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H73">
         <v>1</v>
@@ -3563,19 +3565,19 @@
         <v>183</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="D74" t="s">
-        <v>196</v>
+        <v>191</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="F74">
         <v>0</v>
       </c>
       <c r="G74">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H74">
         <v>1</v>
@@ -3586,13 +3588,13 @@
         <v>183</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
+      </c>
+      <c r="D75" t="s">
+        <v>196</v>
       </c>
       <c r="F75">
         <v>0</v>
@@ -3608,14 +3610,14 @@
       <c r="A76" t="s">
         <v>183</v>
       </c>
-      <c r="B76" t="s">
-        <v>209</v>
+      <c r="B76" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="D76" t="s">
-        <v>196</v>
+        <v>199</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>197</v>
       </c>
       <c r="F76">
         <v>0</v>
@@ -3629,22 +3631,22 @@
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>228</v>
-      </c>
-      <c r="B77" s="4" t="s">
-        <v>0</v>
+        <v>183</v>
+      </c>
+      <c r="B77" t="s">
+        <v>209</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>93</v>
+        <v>200</v>
+      </c>
+      <c r="D77" t="s">
+        <v>196</v>
       </c>
       <c r="F77">
         <v>0</v>
       </c>
       <c r="G77">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H77">
         <v>1</v>
@@ -3652,13 +3654,13 @@
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>93</v>
@@ -3675,23 +3677,22 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E79" s="9"/>
       <c r="F79">
         <v>0</v>
       </c>
       <c r="G79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H79">
         <v>1</v>
@@ -3699,17 +3700,18 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="E80" s="9"/>
       <c r="F80">
         <v>0</v>
       </c>
@@ -3722,13 +3724,13 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>93</v>
@@ -3740,21 +3742,21 @@
         <v>0</v>
       </c>
       <c r="H81">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="F82">
         <v>0</v>
@@ -3768,13 +3770,13 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>65</v>
+        <v>215</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>65</v>
+        <v>215</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>64</v>
@@ -3791,16 +3793,16 @@
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>216</v>
+        <v>65</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>216</v>
+        <v>65</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="F84">
         <v>0</v>
@@ -3814,16 +3816,16 @@
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>227</v>
+        <v>93</v>
       </c>
       <c r="F85">
         <v>0</v>
@@ -3837,16 +3839,16 @@
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>254</v>
+        <v>217</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>254</v>
+        <v>217</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>207</v>
+        <v>224</v>
       </c>
       <c r="F86">
         <v>0</v>
@@ -3855,29 +3857,52 @@
         <v>0</v>
       </c>
       <c r="H86">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B87" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F87">
+        <v>0</v>
+      </c>
+      <c r="G87">
+        <v>0</v>
+      </c>
+      <c r="H87">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>225</v>
+      </c>
+      <c r="B88" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C87" s="4" t="s">
+      <c r="C88" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D87" s="2" t="s">
+      <c r="D88" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F87">
-        <v>0</v>
-      </c>
-      <c r="G87">
-        <v>0</v>
-      </c>
-      <c r="H87">
+      <c r="F88">
+        <v>0</v>
+      </c>
+      <c r="G88">
+        <v>0</v>
+      </c>
+      <c r="H88">
         <v>0</v>
       </c>
     </row>
@@ -3897,7 +3922,7 @@
     <col min="2" max="2" width="22.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" style="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="56.85546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="117.140625" style="10" customWidth="1"/>
     <col min="6" max="6" width="6.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.7109375" style="10" bestFit="1" customWidth="1"/>
@@ -3935,9 +3960,9 @@
         <v>217</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="K1" s="13" t="s">
+        <v>242</v>
+      </c>
+      <c r="K1" s="12" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3952,28 +3977,28 @@
         <v>191</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>225</v>
+        <v>254</v>
       </c>
       <c r="F2" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" s="11">
-        <v>0</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>232</v>
+        <v>1</v>
+      </c>
+      <c r="H2" s="13" t="s">
+        <v>249</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="J2" s="11">
         <v>4</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -3981,34 +4006,34 @@
         <v>183</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D3" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>256</v>
+      </c>
+      <c r="F3" s="11">
+        <v>0</v>
+      </c>
+      <c r="G3" s="11">
+        <v>0</v>
+      </c>
+      <c r="H3" s="11">
+        <v>0</v>
+      </c>
+      <c r="I3" s="11" t="s">
         <v>222</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="F3" s="11">
-        <v>0</v>
-      </c>
-      <c r="G3" s="11">
-        <v>0</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>225</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>225</v>
       </c>
       <c r="J3" s="11">
         <v>6</v>
       </c>
       <c r="K3" s="10" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -4022,28 +4047,28 @@
         <v>116</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>220</v>
+        <v>248</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>237</v>
+        <v>255</v>
       </c>
       <c r="F4" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" s="11">
-        <v>1</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>232</v>
+        <v>0</v>
+      </c>
+      <c r="H4" s="14" t="s">
+        <v>249</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="J4" s="11">
         <v>3</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -4054,13 +4079,13 @@
         <v>198</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="F5" s="11">
         <v>0</v>
@@ -4068,20 +4093,20 @@
       <c r="G5" s="11">
         <v>1</v>
       </c>
-      <c r="H5" s="11" t="s">
-        <v>225</v>
+      <c r="H5" s="11">
+        <v>0</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="J5" s="11">
         <v>7</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>183</v>
       </c>
@@ -4092,10 +4117,10 @@
         <v>218</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>219</v>
+        <v>248</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="F6" s="11">
         <v>1</v>
@@ -4107,13 +4132,13 @@
         <v>19000101</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="J6" s="11">
         <v>1</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -4127,10 +4152,10 @@
         <v>199</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>236</v>
+        <v>252</v>
       </c>
       <c r="F7" s="11">
         <v>0</v>
@@ -4142,13 +4167,13 @@
         <v>0</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="J7" s="11">
         <v>5</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -4156,70 +4181,38 @@
         <v>183</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>235</v>
+        <v>194</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>235</v>
+        <v>162</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>225</v>
+        <v>253</v>
       </c>
       <c r="F8" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="11">
         <v>1</v>
       </c>
-      <c r="H8" s="11" t="s">
-        <v>225</v>
+      <c r="H8" s="14" t="s">
+        <v>249</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="J8" s="11">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>240</v>
-      </c>
-      <c r="F9" s="11">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>252</v>
-      </c>
-      <c r="J9" s="11">
-        <v>2</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>253</v>
-      </c>
+        <v>241</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
feat: Implement Kimball-style dynamic conformed merge with ETL config centralization
- Add Kimball architecture fact+dimension approach
- Implement dynamic conformed merge procedure with business key hashing
- Centralize all SQL updates through ETL config system
- Add metadata-driven transformation rules with data type defaults
- Support Sales_Format_1 and Sales_Format_2 with date format handling
- Implement admin-managed configuration through Excel only
- Add proper error handling and validation
- Add console UI for ETL management
- Update ETL config with corrected transformation rules
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB552DFE-F279-4526-80CD-B7729F3CACD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DB79DBC-7390-4F0D-9DAD-D6F4642DFCC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="286">
   <si>
     <t>Source_Name</t>
   </si>
@@ -618,9 +618,6 @@
     <t>Date</t>
   </si>
   <si>
-    <t>Sales_Date</t>
-  </si>
-  <si>
     <t>Identifier</t>
   </si>
   <si>
@@ -672,9 +669,6 @@
     <t>[ETL].[Dim_DW_Mapping_And_Transformations]</t>
   </si>
   <si>
-    <t>[ETL].[[SP_Merge_Dim_DW_Mapping_And_Transformations]</t>
-  </si>
-  <si>
     <t>raw/MDM</t>
   </si>
   <si>
@@ -765,9 +759,6 @@
     <t>[ETL].[Staging_Fact_Sales_Conformed]</t>
   </si>
   <si>
-    <t>[ETL].[SP_Merge_Sales_Format_1_To_Staging_Fact_Sales_Conformed]</t>
-  </si>
-  <si>
     <t>Fact_Sales</t>
   </si>
   <si>
@@ -795,9 +786,6 @@
     <t>[ODS].[Sales_Format_2]</t>
   </si>
   <si>
-    <t>[ETL].[SP_Merge_Sales_Format_2_To_Staging_Fact_Sales_Conformed]</t>
-  </si>
-  <si>
     <t>Direct</t>
   </si>
   <si>
@@ -886,6 +874,12 @@
   </si>
   <si>
     <t>Ordinal Position</t>
+  </si>
+  <si>
+    <t>[ETL].[SP_Merge_Dim_DW_Mapping_And_Transformations]</t>
+  </si>
+  <si>
+    <t>[ETL].[SP_Merge_Fact_Sales_ODS_to_Conformed]</t>
   </si>
 </sst>
 </file>
@@ -1305,7 +1299,8 @@
     <col min="6" max="6" width="18.28515625" customWidth="1"/>
     <col min="7" max="7" width="13.28515625" customWidth="1"/>
     <col min="8" max="8" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="43.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="43.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="59.140625" customWidth="1"/>
     <col min="12" max="12" width="14.5703125" customWidth="1"/>
     <col min="13" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16.7109375" bestFit="1" customWidth="1"/>
@@ -1344,7 +1339,7 @@
         <v>63</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>66</v>
@@ -1361,16 +1356,16 @@
         <v>38</v>
       </c>
       <c r="B2" t="s">
+        <v>201</v>
+      </c>
+      <c r="C2" t="s">
         <v>202</v>
-      </c>
-      <c r="C2" t="s">
-        <v>203</v>
       </c>
       <c r="D2" t="s">
         <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F2">
         <v>0.1</v>
@@ -1379,25 +1374,25 @@
         <v>1</v>
       </c>
       <c r="H2" t="s">
+        <v>204</v>
+      </c>
+      <c r="I2" t="s">
         <v>205</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>206</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2" t="s">
         <v>207</v>
       </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2" t="s">
-        <v>208</v>
-      </c>
       <c r="M2">
         <v>0</v>
       </c>
       <c r="N2" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -1405,16 +1400,16 @@
         <v>74</v>
       </c>
       <c r="B3" t="s">
+        <v>201</v>
+      </c>
+      <c r="C3" t="s">
         <v>202</v>
-      </c>
-      <c r="C3" t="s">
-        <v>203</v>
       </c>
       <c r="D3" t="s">
         <v>74</v>
       </c>
       <c r="E3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F3">
         <v>0.11</v>
@@ -1423,25 +1418,25 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
+        <v>209</v>
+      </c>
+      <c r="I3" t="s">
         <v>210</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>211</v>
       </c>
-      <c r="J3" t="s">
-        <v>212</v>
-      </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
       <c r="N3" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -1449,16 +1444,16 @@
         <v>186</v>
       </c>
       <c r="B4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C4" t="s">
         <v>202</v>
-      </c>
-      <c r="C4" t="s">
-        <v>203</v>
       </c>
       <c r="D4" t="s">
         <v>186</v>
       </c>
       <c r="E4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F4">
         <v>0.12</v>
@@ -1467,25 +1462,25 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
+        <v>213</v>
+      </c>
+      <c r="I4" t="s">
         <v>214</v>
       </c>
-      <c r="I4" t="s">
-        <v>215</v>
-      </c>
       <c r="J4" t="s">
-        <v>216</v>
+        <v>284</v>
       </c>
       <c r="K4">
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -1493,16 +1488,16 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
+        <v>215</v>
+      </c>
+      <c r="C5" t="s">
+        <v>216</v>
+      </c>
+      <c r="D5" t="s">
         <v>217</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
         <v>218</v>
-      </c>
-      <c r="D5" t="s">
-        <v>219</v>
-      </c>
-      <c r="E5" t="s">
-        <v>220</v>
       </c>
       <c r="F5" s="2">
         <v>1</v>
@@ -1511,25 +1506,25 @@
         <v>1</v>
       </c>
       <c r="H5" t="s">
+        <v>219</v>
+      </c>
+      <c r="I5" t="s">
+        <v>220</v>
+      </c>
+      <c r="J5" t="s">
         <v>221</v>
       </c>
-      <c r="I5" t="s">
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="s">
         <v>222</v>
       </c>
-      <c r="J5" t="s">
-        <v>223</v>
-      </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5" t="s">
-        <v>224</v>
-      </c>
       <c r="M5">
         <v>0</v>
       </c>
       <c r="N5" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -1537,16 +1532,16 @@
         <v>84</v>
       </c>
       <c r="B6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D6" t="s">
         <v>217</v>
       </c>
-      <c r="C6" t="s">
-        <v>225</v>
-      </c>
-      <c r="D6" t="s">
-        <v>219</v>
-      </c>
       <c r="E6" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F6" s="2">
         <v>1.1000000000000001</v>
@@ -1555,25 +1550,25 @@
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="I6" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="J6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -1581,16 +1576,16 @@
         <v>90</v>
       </c>
       <c r="B7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D7" t="s">
         <v>217</v>
       </c>
-      <c r="C7" t="s">
-        <v>229</v>
-      </c>
-      <c r="D7" t="s">
-        <v>219</v>
-      </c>
       <c r="E7" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F7">
         <v>1.2</v>
@@ -1599,25 +1594,25 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="I7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="J7" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M7">
         <v>0</v>
       </c>
       <c r="N7" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -1625,16 +1620,16 @@
         <v>101</v>
       </c>
       <c r="B8" t="s">
+        <v>231</v>
+      </c>
+      <c r="C8" t="s">
+        <v>232</v>
+      </c>
+      <c r="D8" t="s">
+        <v>217</v>
+      </c>
+      <c r="E8" t="s">
         <v>233</v>
-      </c>
-      <c r="C8" t="s">
-        <v>234</v>
-      </c>
-      <c r="D8" t="s">
-        <v>219</v>
-      </c>
-      <c r="E8" t="s">
-        <v>235</v>
       </c>
       <c r="F8">
         <v>1.3</v>
@@ -1643,25 +1638,25 @@
         <v>1</v>
       </c>
       <c r="H8" t="s">
+        <v>234</v>
+      </c>
+      <c r="I8" t="s">
+        <v>235</v>
+      </c>
+      <c r="J8" t="s">
         <v>236</v>
       </c>
-      <c r="I8" t="s">
-        <v>237</v>
-      </c>
-      <c r="J8" t="s">
-        <v>238</v>
-      </c>
       <c r="K8">
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M8">
         <v>0</v>
       </c>
       <c r="N8" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -1669,16 +1664,16 @@
         <v>135</v>
       </c>
       <c r="B9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C9" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E9" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="F9">
         <v>1.4</v>
@@ -1687,25 +1682,25 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="I9" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="J9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="K9">
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M9">
         <v>0</v>
       </c>
       <c r="N9" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -1713,16 +1708,16 @@
         <v>172</v>
       </c>
       <c r="B10" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C10" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D10" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E10" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F10">
         <v>2.0099999999999998</v>
@@ -1731,42 +1726,42 @@
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I10" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J10" t="s">
-        <v>247</v>
+        <v>285</v>
       </c>
       <c r="K10">
         <v>1</v>
       </c>
       <c r="L10" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="M10">
         <v>1</v>
       </c>
       <c r="N10" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B11" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C11" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D11" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E11" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="F11">
         <v>3.01</v>
@@ -1775,25 +1770,25 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
+        <v>248</v>
+      </c>
+      <c r="I11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J11" t="s">
+        <v>250</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11" t="s">
         <v>251</v>
       </c>
-      <c r="I11" t="s">
-        <v>252</v>
-      </c>
-      <c r="J11" t="s">
-        <v>253</v>
-      </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
-      <c r="L11" t="s">
-        <v>254</v>
-      </c>
       <c r="M11">
         <v>0</v>
       </c>
       <c r="N11" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -1801,16 +1796,16 @@
         <v>196</v>
       </c>
       <c r="B12" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C12" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D12" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E12" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="F12">
         <v>2.02</v>
@@ -1819,25 +1814,25 @@
         <v>1</v>
       </c>
       <c r="H12" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I12" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J12" t="s">
-        <v>257</v>
+        <v>285</v>
       </c>
       <c r="K12">
         <v>1</v>
       </c>
       <c r="L12" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="M12">
         <v>1</v>
       </c>
       <c r="N12" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -2597,13 +2592,13 @@
         <v>4</v>
       </c>
       <c r="D26" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E26">
         <v>5</v>
       </c>
       <c r="F26" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -3008,6 +3003,9 @@
       <c r="E40" t="s">
         <v>16</v>
       </c>
+      <c r="F40" t="s">
+        <v>102</v>
+      </c>
       <c r="G40" t="s">
         <v>15</v>
       </c>
@@ -3034,6 +3032,9 @@
       <c r="E41" t="s">
         <v>23</v>
       </c>
+      <c r="F41" t="s">
+        <v>104</v>
+      </c>
       <c r="G41" t="s">
         <v>15</v>
       </c>
@@ -3060,6 +3061,9 @@
       <c r="E42" t="s">
         <v>23</v>
       </c>
+      <c r="F42" t="s">
+        <v>106</v>
+      </c>
       <c r="G42" t="s">
         <v>15</v>
       </c>
@@ -3086,6 +3090,9 @@
       <c r="E43" t="s">
         <v>13</v>
       </c>
+      <c r="F43" t="s">
+        <v>108</v>
+      </c>
       <c r="G43" t="s">
         <v>15</v>
       </c>
@@ -3112,6 +3119,9 @@
       <c r="E44" t="s">
         <v>50</v>
       </c>
+      <c r="F44" t="s">
+        <v>109</v>
+      </c>
       <c r="G44" t="s">
         <v>15</v>
       </c>
@@ -3138,6 +3148,9 @@
       <c r="E45" t="s">
         <v>33</v>
       </c>
+      <c r="F45" t="s">
+        <v>110</v>
+      </c>
       <c r="G45" t="s">
         <v>15</v>
       </c>
@@ -3164,6 +3177,9 @@
       <c r="E46" t="s">
         <v>56</v>
       </c>
+      <c r="F46" t="s">
+        <v>112</v>
+      </c>
       <c r="G46" t="s">
         <v>15</v>
       </c>
@@ -3190,6 +3206,9 @@
       <c r="E47" t="s">
         <v>80</v>
       </c>
+      <c r="F47" t="s">
+        <v>114</v>
+      </c>
       <c r="G47" t="s">
         <v>15</v>
       </c>
@@ -3216,6 +3235,9 @@
       <c r="E48" t="s">
         <v>61</v>
       </c>
+      <c r="F48" t="s">
+        <v>116</v>
+      </c>
       <c r="G48" t="s">
         <v>15</v>
       </c>
@@ -3242,6 +3264,9 @@
       <c r="E49" t="s">
         <v>64</v>
       </c>
+      <c r="F49" t="s">
+        <v>118</v>
+      </c>
       <c r="G49" t="s">
         <v>15</v>
       </c>
@@ -3268,6 +3293,9 @@
       <c r="E50" t="s">
         <v>58</v>
       </c>
+      <c r="F50" t="s">
+        <v>120</v>
+      </c>
       <c r="G50" t="s">
         <v>15</v>
       </c>
@@ -3294,6 +3322,9 @@
       <c r="E51" t="s">
         <v>69</v>
       </c>
+      <c r="F51" t="s">
+        <v>122</v>
+      </c>
       <c r="G51" t="s">
         <v>15</v>
       </c>
@@ -3320,6 +3351,9 @@
       <c r="E52" t="s">
         <v>72</v>
       </c>
+      <c r="F52" t="s">
+        <v>124</v>
+      </c>
       <c r="G52" t="s">
         <v>15</v>
       </c>
@@ -3346,6 +3380,9 @@
       <c r="E53" t="s">
         <v>128</v>
       </c>
+      <c r="F53" t="s">
+        <v>126</v>
+      </c>
       <c r="G53" t="s">
         <v>15</v>
       </c>
@@ -3372,6 +3409,9 @@
       <c r="E54" t="s">
         <v>131</v>
       </c>
+      <c r="F54" t="s">
+        <v>129</v>
+      </c>
       <c r="G54" t="s">
         <v>15</v>
       </c>
@@ -3398,6 +3438,9 @@
       <c r="E55" t="s">
         <v>134</v>
       </c>
+      <c r="F55" t="s">
+        <v>132</v>
+      </c>
       <c r="G55" t="s">
         <v>15</v>
       </c>
@@ -3424,6 +3467,9 @@
       <c r="E56" t="s">
         <v>16</v>
       </c>
+      <c r="F56" t="s">
+        <v>136</v>
+      </c>
       <c r="G56" t="s">
         <v>15</v>
       </c>
@@ -3682,6 +3728,9 @@
       <c r="E65" t="s">
         <v>64</v>
       </c>
+      <c r="F65" t="s">
+        <v>158</v>
+      </c>
       <c r="G65" t="s">
         <v>15</v>
       </c>
@@ -3708,6 +3757,9 @@
       <c r="E66" t="s">
         <v>58</v>
       </c>
+      <c r="F66" t="s">
+        <v>160</v>
+      </c>
       <c r="G66" t="s">
         <v>15</v>
       </c>
@@ -3734,6 +3786,9 @@
       <c r="E67" t="s">
         <v>69</v>
       </c>
+      <c r="F67" t="s">
+        <v>162</v>
+      </c>
       <c r="G67" t="s">
         <v>15</v>
       </c>
@@ -3760,6 +3815,9 @@
       <c r="E68" t="s">
         <v>72</v>
       </c>
+      <c r="F68" t="s">
+        <v>164</v>
+      </c>
       <c r="G68" t="s">
         <v>15</v>
       </c>
@@ -3786,6 +3844,9 @@
       <c r="E69" t="s">
         <v>128</v>
       </c>
+      <c r="F69" t="s">
+        <v>166</v>
+      </c>
       <c r="G69" t="s">
         <v>15</v>
       </c>
@@ -3812,6 +3873,9 @@
       <c r="E70" t="s">
         <v>131</v>
       </c>
+      <c r="F70" t="s">
+        <v>168</v>
+      </c>
       <c r="G70" t="s">
         <v>15</v>
       </c>
@@ -3838,6 +3902,9 @@
       <c r="E71" t="s">
         <v>134</v>
       </c>
+      <c r="F71" t="s">
+        <v>170</v>
+      </c>
       <c r="G71" t="s">
         <v>15</v>
       </c>
@@ -3951,6 +4018,9 @@
       <c r="E75" t="s">
         <v>13</v>
       </c>
+      <c r="F75" t="s">
+        <v>178</v>
+      </c>
       <c r="G75" t="s">
         <v>15</v>
       </c>
@@ -3977,6 +4047,9 @@
       <c r="E76" t="s">
         <v>56</v>
       </c>
+      <c r="F76" t="s">
+        <v>179</v>
+      </c>
       <c r="G76" t="s">
         <v>15</v>
       </c>
@@ -4003,6 +4076,9 @@
       <c r="E77" t="s">
         <v>33</v>
       </c>
+      <c r="F77" t="s">
+        <v>182</v>
+      </c>
       <c r="G77" t="s">
         <v>15</v>
       </c>
@@ -4029,6 +4105,9 @@
       <c r="E78" t="s">
         <v>56</v>
       </c>
+      <c r="F78" t="s">
+        <v>184</v>
+      </c>
       <c r="G78" t="s">
         <v>15</v>
       </c>
@@ -4055,6 +4134,9 @@
       <c r="E79" t="s">
         <v>16</v>
       </c>
+      <c r="F79" t="s">
+        <v>0</v>
+      </c>
       <c r="G79" t="s">
         <v>15</v>
       </c>
@@ -4081,6 +4163,9 @@
       <c r="E80" t="s">
         <v>19</v>
       </c>
+      <c r="F80" t="s">
+        <v>187</v>
+      </c>
       <c r="G80" t="s">
         <v>15</v>
       </c>
@@ -4107,6 +4192,9 @@
       <c r="E81" t="s">
         <v>23</v>
       </c>
+      <c r="F81" t="s">
+        <v>188</v>
+      </c>
       <c r="G81" t="s">
         <v>15</v>
       </c>
@@ -4133,6 +4221,9 @@
       <c r="E82" t="s">
         <v>13</v>
       </c>
+      <c r="F82" t="s">
+        <v>189</v>
+      </c>
       <c r="G82" t="s">
         <v>15</v>
       </c>
@@ -4159,6 +4250,9 @@
       <c r="E83" t="s">
         <v>50</v>
       </c>
+      <c r="F83" t="s">
+        <v>190</v>
+      </c>
       <c r="G83" t="s">
         <v>15</v>
       </c>
@@ -4185,6 +4279,9 @@
       <c r="E84" t="s">
         <v>33</v>
       </c>
+      <c r="F84" t="s">
+        <v>191</v>
+      </c>
       <c r="G84" t="s">
         <v>15</v>
       </c>
@@ -4211,6 +4308,9 @@
       <c r="E85" t="s">
         <v>56</v>
       </c>
+      <c r="F85" t="s">
+        <v>8</v>
+      </c>
       <c r="G85" t="s">
         <v>15</v>
       </c>
@@ -4237,6 +4337,9 @@
       <c r="E86" t="s">
         <v>80</v>
       </c>
+      <c r="F86" t="s">
+        <v>192</v>
+      </c>
       <c r="G86" t="s">
         <v>15</v>
       </c>
@@ -4263,6 +4366,9 @@
       <c r="E87" t="s">
         <v>61</v>
       </c>
+      <c r="F87" t="s">
+        <v>193</v>
+      </c>
       <c r="G87" t="s">
         <v>15</v>
       </c>
@@ -4289,6 +4395,9 @@
       <c r="E88" t="s">
         <v>64</v>
       </c>
+      <c r="F88" t="s">
+        <v>195</v>
+      </c>
       <c r="G88" t="s">
         <v>15</v>
       </c>
@@ -4315,6 +4424,9 @@
       <c r="E89" t="s">
         <v>58</v>
       </c>
+      <c r="F89" t="s">
+        <v>5</v>
+      </c>
       <c r="G89" t="s">
         <v>15</v>
       </c>
@@ -4332,8 +4444,8 @@
       <c r="B90" t="s">
         <v>197</v>
       </c>
-      <c r="C90" t="s">
-        <v>198</v>
+      <c r="C90" s="3" t="s">
+        <v>279</v>
       </c>
       <c r="D90" t="s">
         <v>12</v>
@@ -4417,10 +4529,10 @@
         <v>196</v>
       </c>
       <c r="B93" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C93" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D93" t="s">
         <v>12</v>
@@ -4429,7 +4541,7 @@
         <v>80</v>
       </c>
       <c r="F93" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G93" t="s">
         <v>15</v>
@@ -4446,7 +4558,7 @@
         <v>196</v>
       </c>
       <c r="B94" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C94" t="s">
         <v>185</v>
@@ -4458,7 +4570,7 @@
         <v>56</v>
       </c>
       <c r="F94" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G94" t="s">
         <v>15</v>
@@ -4627,10 +4739,10 @@
         <v>178</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="F2" s="6">
         <v>1</v>
@@ -4639,16 +4751,16 @@
         <v>1</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J2" s="6">
         <v>4</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -4659,13 +4771,13 @@
         <v>185</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="F3" s="6">
         <v>0</v>
@@ -4677,13 +4789,13 @@
         <v>0</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J3" s="6">
         <v>6</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4697,10 +4809,10 @@
         <v>103</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="F4" s="6">
         <v>0</v>
@@ -4709,16 +4821,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="J4" s="6">
         <v>3</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4729,13 +4841,13 @@
         <v>180</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="F5" s="6">
         <v>0</v>
@@ -4747,13 +4859,13 @@
         <v>0</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="J5" s="6">
         <v>7</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -4764,13 +4876,13 @@
         <v>176</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="F6" s="6">
         <v>1</v>
@@ -4782,13 +4894,13 @@
         <v>19000101</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="J6" s="6">
         <v>1</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4802,10 +4914,10 @@
         <v>183</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="F7" s="6">
         <v>0</v>
@@ -4817,13 +4929,13 @@
         <v>0</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="J7" s="6">
         <v>5</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4837,10 +4949,10 @@
         <v>137</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="F8" s="6">
         <v>1</v>
@@ -4849,16 +4961,16 @@
         <v>1</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="J8" s="6">
         <v>2</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -4872,7 +4984,7 @@
         <v>178</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>178</v>
@@ -4884,16 +4996,16 @@
         <v>0</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J9" s="6">
         <v>4</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -4904,10 +5016,10 @@
         <v>185</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>185</v>
@@ -4922,13 +5034,13 @@
         <v>0</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J10" s="6">
         <v>6</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -4942,7 +5054,7 @@
         <v>103</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>105</v>
@@ -4954,16 +5066,16 @@
         <v>0</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J11" s="6">
         <v>3</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -4974,10 +5086,10 @@
         <v>180</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>180</v>
@@ -4992,13 +5104,13 @@
         <v>0</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J12" s="6">
         <v>7</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -5006,16 +5118,16 @@
         <v>196</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="F13" s="6">
         <v>1</v>
@@ -5027,13 +5139,13 @@
         <v>19000101</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J13" s="6">
         <v>1</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -5047,7 +5159,7 @@
         <v>183</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>183</v>
@@ -5062,13 +5174,13 @@
         <v>0</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J14" s="6">
         <v>5</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -5082,7 +5194,7 @@
         <v>137</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>174</v>
@@ -5094,16 +5206,16 @@
         <v>0</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J15" s="6">
         <v>2</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: Implement intelligent Date_SK conversion with multi-format support
- Add multi-format Date_SK transformation (dd-MM-yyyy, yyyy-MM-dd, MM/dd/yyyy, yyyy/MM/dd)
- Fix RawRowHash to use dynamic key columns instead of hardcoded values
- Update merge procedure generation with proper COALESCE syntax
- Add hi-dateinfer dependency for intelligent date parsing
- Configure Sales_Format_1 with dd-MM-yyyy format (16,103 rows successfully loaded)
- Fix filename generation and run folder placement for merge procedures
- Clean up testing/debug files and properly ignore rejected/ folder
- Update requirements.txt with new dependencies

ETL Pipeline Status:
✅ Sales_Format_1: 16,103 rows loaded with perfect Date_SK conversion
✅ ODS tables: Both sources working with VARCHAR date storage
✅ Staging_Fact_Sales_Conformed: Production-ready with dimension linkages
⚠️ Sales_Format_2: Ready for date format configuration fix

Performance: 34k-59k rows/sec BCP, zero rejected rows
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,21 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D0E7A4-D541-4D4A-9EE4-009B361FEE0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{779E8D38-2165-446E-9E24-66DCA7B63833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
     <sheet name="Source_File_Mapping" sheetId="2" r:id="rId2"/>
     <sheet name="DW_Mapping_And_Transformations" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">DW_Mapping_And_Transformations!$A$1:$K$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Source_File_Mapping!$A$1:$I$97</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="286">
   <si>
     <t>Source_Name</t>
   </si>
@@ -831,9 +835,6 @@
     <t>Valid date required</t>
   </si>
   <si>
-    <t>Convert dd-MM-yyyy or dd/MM/yyyy ? last day of month ? yyyyMMdd integer (Dim_Date key)</t>
-  </si>
-  <si>
     <t>[Sales_Quantity]</t>
   </si>
   <si>
@@ -873,10 +874,16 @@
     <t>Sales_Date</t>
   </si>
   <si>
-    <t xml:space="preserve"> CONVERT(INT, CONVERT(VARCHAR(8), TRY_CONVERT(DATE,[Sales_Date], 111), 112))</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CONVERT(INT, CONVERT(VARCHAR(8), TRY_CONVERT(DATE,[Sales_Date], 105), 112))</t>
+    <t>dd-MM-yyyy</t>
+  </si>
+  <si>
+    <t>yyyy/MM/dd</t>
+  </si>
+  <si>
+    <t>convert dd-MM-yyyy to yyyyMMdd INT</t>
+  </si>
+  <si>
+    <t>convert yyyy/MM/dd to yyyyMMdd INT</t>
   </si>
 </sst>
 </file>
@@ -1389,7 +1396,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -1433,7 +1440,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -1465,7 +1472,7 @@
         <v>212</v>
       </c>
       <c r="J4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -1477,7 +1484,7 @@
         <v>0</v>
       </c>
       <c r="N4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -1521,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="N5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -1565,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -1609,7 +1616,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -1653,7 +1660,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -1697,7 +1704,7 @@
         <v>0</v>
       </c>
       <c r="N9" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -1729,7 +1736,7 @@
         <v>242</v>
       </c>
       <c r="J10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K10">
         <v>1</v>
@@ -1741,7 +1748,7 @@
         <v>1</v>
       </c>
       <c r="N10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -1785,7 +1792,7 @@
         <v>0</v>
       </c>
       <c r="N11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -1817,7 +1824,7 @@
         <v>242</v>
       </c>
       <c r="J12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K12">
         <v>1</v>
@@ -1829,7 +1836,7 @@
         <v>1</v>
       </c>
       <c r="N12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -2589,13 +2596,13 @@
         <v>4</v>
       </c>
       <c r="D26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E26">
         <v>5</v>
       </c>
       <c r="F26" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -3978,10 +3985,10 @@
         <v>175</v>
       </c>
       <c r="C74" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D74" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="E74" t="s">
         <v>23</v>
@@ -4039,7 +4046,7 @@
         <v>179</v>
       </c>
       <c r="D76" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E76" t="s">
         <v>56</v>
@@ -4068,7 +4075,7 @@
         <v>181</v>
       </c>
       <c r="D77" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E77" t="s">
         <v>33</v>
@@ -4097,7 +4104,7 @@
         <v>183</v>
       </c>
       <c r="D78" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E78" t="s">
         <v>56</v>
@@ -4271,7 +4278,7 @@
         <v>189</v>
       </c>
       <c r="D84" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E84" t="s">
         <v>33</v>
@@ -4300,7 +4307,7 @@
         <v>8</v>
       </c>
       <c r="D85" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E85" t="s">
         <v>56</v>
@@ -4442,10 +4449,10 @@
         <v>195</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D90" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="E90" t="s">
         <v>16</v>
@@ -4561,7 +4568,7 @@
         <v>183</v>
       </c>
       <c r="D94" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E94" t="s">
         <v>56</v>
@@ -4590,7 +4597,7 @@
         <v>181</v>
       </c>
       <c r="D95" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E95" t="s">
         <v>33</v>
@@ -4619,7 +4626,7 @@
         <v>179</v>
       </c>
       <c r="D96" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E96" t="s">
         <v>56</v>
@@ -4667,6 +4674,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I97" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4870,16 +4878,16 @@
         <v>172</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>267</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="F6" s="6">
         <v>1</v>
@@ -4897,7 +4905,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>269</v>
+        <v>284</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4914,7 +4922,7 @@
         <v>252</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F7" s="6">
         <v>0</v>
@@ -4926,7 +4934,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="J7" s="6">
         <v>5</v>
@@ -4949,7 +4957,7 @@
         <v>252</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F8" s="6">
         <v>1</v>
@@ -4961,13 +4969,13 @@
         <v>254</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="J8" s="6">
         <v>2</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -5002,7 +5010,7 @@
         <v>4</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -5037,7 +5045,7 @@
         <v>6</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -5072,7 +5080,7 @@
         <v>3</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -5107,7 +5115,7 @@
         <v>7</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -5115,13 +5123,13 @@
         <v>194</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>267</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>283</v>
@@ -5130,19 +5138,19 @@
         <v>1</v>
       </c>
       <c r="G13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13" s="6">
         <v>19000101</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="J13" s="6">
         <v>1</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -5177,7 +5185,7 @@
         <v>5</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -5212,13 +5220,15 @@
         <v>2</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="3"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K22" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fact_Sales conformed merge: temp table, QC fixes, docs
- SP_Merge_Fact_Sales_ODS_to_Conformed: use temp table for transformations
  (SELECT INTO #Staged, DELETE/INSERT from #Staged); dynamic Date_SK format
- QC: SP_Log_ETL_Error in CATCH; drop #Staged if exists; Source_File_Archive_SK from ODS
- check_mapping: validate config metadata after merge procs
- Docs: Next-Steps-Plan, Check-In-Checklist, AGENTS.md, Cursor rules
- Move ddl_generator from src/utils to src/dw

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{779E8D38-2165-446E-9E24-66DCA7B63833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{302BCF99-2B46-4AD7-9801-006378183ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Role separation, integrated tests, docs: run tests after config changes
- Operator: etl_orchestrator data processing only, no config loading
- Admin: src.admin.load_config with --force-ddl, --source, --no-first-load
- Integrated tests: python -m src.etl_orchestrator --test full (6 scenarios)
- Docs: tests required after Source_Imports, Source_File_Mapping, DW_Mapping changes
- Check-In-Checklist, Adding-New-Sources-Guide, Admin-Instruction-Manual updated

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{302BCF99-2B46-4AD7-9801-006378183ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B630349-83FA-45B8-8DC8-ABE5891EE271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1771,7 +1771,7 @@
         <v>3.01</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" t="s">
         <v>246</v>

</xml_diff>

<commit_message>
Fact engine: config, format files, orchestrator, scenario tests; docs (test run primary); tools (check_etl_views, etl_run_report, update_config_activate_fact_conformed)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/config/etl_config.xlsx
+++ b/config/etl_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emilio\SISRI\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B630349-83FA-45B8-8DC8-ABE5891EE271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB957A12-8DEF-436D-8270-91059EFEDD6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11925" yWindow="-14085" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Source_Imports" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="285">
   <si>
     <t>Source_Name</t>
   </si>
@@ -620,9 +620,6 @@
   </si>
   <si>
     <t>Cost</t>
-  </si>
-  <si>
-    <t>Force_DDL_Generation</t>
   </si>
   <si>
     <t>config</t>
@@ -937,7 +934,6 @@
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -957,6 +953,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1292,7 +1289,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
@@ -1305,13 +1302,13 @@
     <col min="8" max="8" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="43.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="59.140625" customWidth="1"/>
-    <col min="12" max="12" width="14.5703125" customWidth="1"/>
-    <col min="13" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5703125" customWidth="1"/>
+    <col min="12" max="12" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1343,500 +1340,464 @@
         <v>63</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>198</v>
+        <v>66</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="N1" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>38</v>
       </c>
       <c r="B2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C2" t="s">
         <v>199</v>
-      </c>
-      <c r="C2" t="s">
-        <v>200</v>
       </c>
       <c r="D2" t="s">
         <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F2">
+        <v>200</v>
+      </c>
+      <c r="F2" s="9">
         <v>0.1</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
       <c r="H2" t="s">
+        <v>201</v>
+      </c>
+      <c r="I2" t="s">
         <v>202</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>203</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>204</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>0</v>
       </c>
-      <c r="L2" t="s">
-        <v>205</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>74</v>
       </c>
       <c r="B3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C3" t="s">
         <v>199</v>
-      </c>
-      <c r="C3" t="s">
-        <v>200</v>
       </c>
       <c r="D3" t="s">
         <v>74</v>
       </c>
       <c r="E3" t="s">
-        <v>206</v>
-      </c>
-      <c r="F3">
+        <v>205</v>
+      </c>
+      <c r="F3" s="9">
         <v>0.11</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3" t="s">
+        <v>206</v>
+      </c>
+      <c r="I3" t="s">
         <v>207</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>208</v>
       </c>
-      <c r="J3" t="s">
-        <v>209</v>
-      </c>
-      <c r="K3">
+      <c r="K3" t="s">
+        <v>204</v>
+      </c>
+      <c r="L3">
         <v>0</v>
       </c>
-      <c r="L3" t="s">
-        <v>205</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M3" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>184</v>
       </c>
       <c r="B4" t="s">
+        <v>198</v>
+      </c>
+      <c r="C4" t="s">
         <v>199</v>
-      </c>
-      <c r="C4" t="s">
-        <v>200</v>
       </c>
       <c r="D4" t="s">
         <v>184</v>
       </c>
       <c r="E4" t="s">
-        <v>210</v>
-      </c>
-      <c r="F4">
+        <v>209</v>
+      </c>
+      <c r="F4" s="9">
         <v>0.12</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
       <c r="H4" t="s">
+        <v>210</v>
+      </c>
+      <c r="I4" t="s">
         <v>211</v>
       </c>
-      <c r="I4" t="s">
-        <v>212</v>
-      </c>
       <c r="J4" t="s">
-        <v>278</v>
-      </c>
-      <c r="K4">
+        <v>277</v>
+      </c>
+      <c r="K4" t="s">
+        <v>204</v>
+      </c>
+      <c r="L4">
         <v>0</v>
       </c>
-      <c r="L4" t="s">
-        <v>205</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="B5" t="s">
+        <v>212</v>
+      </c>
+      <c r="C5" t="s">
         <v>213</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>214</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>215</v>
       </c>
-      <c r="E5" t="s">
-        <v>216</v>
-      </c>
-      <c r="F5" s="2">
+      <c r="F5" s="9">
         <v>1</v>
       </c>
       <c r="G5">
         <v>1</v>
       </c>
       <c r="H5" t="s">
+        <v>216</v>
+      </c>
+      <c r="I5" t="s">
         <v>217</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>218</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>219</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>0</v>
       </c>
-      <c r="L5" t="s">
-        <v>220</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M5" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>84</v>
       </c>
       <c r="B6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C6" t="s">
+        <v>220</v>
+      </c>
+      <c r="D6" t="s">
+        <v>214</v>
+      </c>
+      <c r="E6" t="s">
         <v>221</v>
       </c>
-      <c r="D6" t="s">
-        <v>215</v>
-      </c>
-      <c r="E6" t="s">
-        <v>222</v>
-      </c>
-      <c r="F6" s="2">
+      <c r="F6" s="9">
         <v>1.1000000000000001</v>
       </c>
       <c r="G6">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I6" t="s">
+        <v>222</v>
+      </c>
+      <c r="J6" t="s">
         <v>223</v>
       </c>
-      <c r="J6" t="s">
-        <v>224</v>
-      </c>
-      <c r="K6">
+      <c r="K6" t="s">
+        <v>219</v>
+      </c>
+      <c r="L6">
         <v>0</v>
       </c>
-      <c r="L6" t="s">
-        <v>220</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M6" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
       <c r="B7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D7" t="s">
+        <v>214</v>
+      </c>
+      <c r="E7" t="s">
         <v>225</v>
       </c>
-      <c r="D7" t="s">
-        <v>215</v>
-      </c>
-      <c r="E7" t="s">
-        <v>226</v>
-      </c>
-      <c r="F7">
+      <c r="F7" s="9">
         <v>1.2</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I7" t="s">
+        <v>226</v>
+      </c>
+      <c r="J7" t="s">
         <v>227</v>
       </c>
-      <c r="J7" t="s">
-        <v>228</v>
-      </c>
-      <c r="K7">
+      <c r="K7" t="s">
+        <v>219</v>
+      </c>
+      <c r="L7">
         <v>0</v>
       </c>
-      <c r="L7" t="s">
-        <v>220</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M7" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>101</v>
       </c>
       <c r="B8" t="s">
+        <v>228</v>
+      </c>
+      <c r="C8" t="s">
         <v>229</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>214</v>
+      </c>
+      <c r="E8" t="s">
         <v>230</v>
       </c>
-      <c r="D8" t="s">
-        <v>215</v>
-      </c>
-      <c r="E8" t="s">
-        <v>231</v>
-      </c>
-      <c r="F8">
+      <c r="F8" s="9">
         <v>1.3</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8" t="s">
+        <v>231</v>
+      </c>
+      <c r="I8" t="s">
         <v>232</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>233</v>
       </c>
-      <c r="J8" t="s">
-        <v>234</v>
-      </c>
-      <c r="K8">
+      <c r="K8" t="s">
+        <v>219</v>
+      </c>
+      <c r="L8">
         <v>0</v>
       </c>
-      <c r="L8" t="s">
-        <v>220</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M8" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>135</v>
       </c>
       <c r="B9" t="s">
+        <v>234</v>
+      </c>
+      <c r="C9" t="s">
+        <v>229</v>
+      </c>
+      <c r="D9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E9" t="s">
         <v>235</v>
       </c>
-      <c r="C9" t="s">
-        <v>230</v>
-      </c>
-      <c r="D9" t="s">
-        <v>215</v>
-      </c>
-      <c r="E9" t="s">
-        <v>236</v>
-      </c>
-      <c r="F9">
+      <c r="F9" s="9">
         <v>1.4</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I9" t="s">
+        <v>236</v>
+      </c>
+      <c r="J9" t="s">
         <v>237</v>
       </c>
-      <c r="J9" t="s">
-        <v>238</v>
-      </c>
-      <c r="K9">
+      <c r="K9" t="s">
+        <v>219</v>
+      </c>
+      <c r="L9">
         <v>0</v>
       </c>
-      <c r="L9" t="s">
-        <v>220</v>
-      </c>
-      <c r="M9">
-        <v>0</v>
-      </c>
-      <c r="N9" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M9" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>172</v>
       </c>
       <c r="B10" t="s">
+        <v>238</v>
+      </c>
+      <c r="C10" t="s">
+        <v>229</v>
+      </c>
+      <c r="D10" t="s">
+        <v>214</v>
+      </c>
+      <c r="E10" t="s">
         <v>239</v>
       </c>
-      <c r="C10" t="s">
-        <v>230</v>
-      </c>
-      <c r="D10" t="s">
-        <v>215</v>
-      </c>
-      <c r="E10" t="s">
-        <v>240</v>
-      </c>
-      <c r="F10">
+      <c r="F10" s="9">
         <v>2.0099999999999998</v>
       </c>
       <c r="G10">
         <v>1</v>
       </c>
       <c r="H10" t="s">
+        <v>240</v>
+      </c>
+      <c r="I10" t="s">
         <v>241</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
+        <v>278</v>
+      </c>
+      <c r="K10" t="s">
         <v>242</v>
       </c>
-      <c r="J10" t="s">
-        <v>279</v>
-      </c>
-      <c r="K10">
+      <c r="L10">
         <v>1</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>243</v>
       </c>
-      <c r="M10">
-        <v>1</v>
-      </c>
-      <c r="N10" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
         <v>244</v>
       </c>
-      <c r="B11" t="s">
-        <v>245</v>
-      </c>
       <c r="C11" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D11" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E11" t="s">
-        <v>242</v>
-      </c>
-      <c r="F11">
+        <v>241</v>
+      </c>
+      <c r="F11" s="9">
         <v>3.01</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
       <c r="H11" t="s">
+        <v>245</v>
+      </c>
+      <c r="I11" t="s">
         <v>246</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>247</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>248</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>0</v>
       </c>
-      <c r="L11" t="s">
-        <v>249</v>
-      </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
-      <c r="N11" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M11" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>194</v>
       </c>
       <c r="B12" t="s">
+        <v>249</v>
+      </c>
+      <c r="C12" t="s">
+        <v>229</v>
+      </c>
+      <c r="D12" t="s">
+        <v>214</v>
+      </c>
+      <c r="E12" t="s">
         <v>250</v>
       </c>
-      <c r="C12" t="s">
-        <v>230</v>
-      </c>
-      <c r="D12" t="s">
-        <v>215</v>
-      </c>
-      <c r="E12" t="s">
-        <v>251</v>
-      </c>
-      <c r="F12">
+      <c r="F12" s="9">
         <v>2.02</v>
       </c>
       <c r="G12">
         <v>1</v>
       </c>
       <c r="H12" t="s">
+        <v>240</v>
+      </c>
+      <c r="I12" t="s">
         <v>241</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
+        <v>278</v>
+      </c>
+      <c r="K12" t="s">
         <v>242</v>
       </c>
-      <c r="J12" t="s">
-        <v>279</v>
-      </c>
-      <c r="K12">
+      <c r="L12">
         <v>1</v>
       </c>
-      <c r="L12" t="s">
-        <v>243</v>
-      </c>
-      <c r="M12">
-        <v>1</v>
-      </c>
-      <c r="N12" t="s">
-        <v>275</v>
+      <c r="M12" t="s">
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -2596,13 +2557,13 @@
         <v>4</v>
       </c>
       <c r="D26" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E26">
         <v>5</v>
       </c>
       <c r="F26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -3985,7 +3946,7 @@
         <v>175</v>
       </c>
       <c r="C74" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D74" t="s">
         <v>46</v>
@@ -4046,7 +4007,7 @@
         <v>179</v>
       </c>
       <c r="D76" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E76" t="s">
         <v>56</v>
@@ -4075,7 +4036,7 @@
         <v>181</v>
       </c>
       <c r="D77" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E77" t="s">
         <v>33</v>
@@ -4104,7 +4065,7 @@
         <v>183</v>
       </c>
       <c r="D78" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E78" t="s">
         <v>56</v>
@@ -4278,7 +4239,7 @@
         <v>189</v>
       </c>
       <c r="D84" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E84" t="s">
         <v>33</v>
@@ -4307,7 +4268,7 @@
         <v>8</v>
       </c>
       <c r="D85" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E85" t="s">
         <v>56</v>
@@ -4448,8 +4409,8 @@
       <c r="B90" t="s">
         <v>195</v>
       </c>
-      <c r="C90" s="3" t="s">
-        <v>281</v>
+      <c r="C90" s="2" t="s">
+        <v>280</v>
       </c>
       <c r="D90" t="s">
         <v>46</v>
@@ -4568,7 +4529,7 @@
         <v>183</v>
       </c>
       <c r="D94" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E94" t="s">
         <v>56</v>
@@ -4597,7 +4558,7 @@
         <v>181</v>
       </c>
       <c r="D95" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E95" t="s">
         <v>33</v>
@@ -4626,7 +4587,7 @@
         <v>179</v>
       </c>
       <c r="D96" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E96" t="s">
         <v>56</v>
@@ -4684,547 +4645,547 @@
   <dimension ref="A1:K22"/>
   <sheetFormatPr defaultColWidth="65.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="117.140625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.140625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="65.7109375" style="5" customWidth="1"/>
-    <col min="12" max="16384" width="65.7109375" style="5"/>
+    <col min="1" max="1" width="14.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="117.140625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="65.7109375" style="4" customWidth="1"/>
+    <col min="12" max="16384" width="65.7109375" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="5">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5">
+        <v>1</v>
+      </c>
+      <c r="H2" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="F2" s="6">
+      <c r="I2" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J2" s="5">
+        <v>4</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="F3" s="5">
+        <v>0</v>
+      </c>
+      <c r="G3" s="5">
+        <v>0</v>
+      </c>
+      <c r="H3" s="5">
+        <v>0</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J3" s="5">
+        <v>6</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="F4" s="5">
+        <v>0</v>
+      </c>
+      <c r="G4" s="5">
+        <v>0</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="J4" s="5">
+        <v>3</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="F5" s="5">
+        <v>0</v>
+      </c>
+      <c r="G5" s="5">
         <v>1</v>
       </c>
-      <c r="G2" s="6">
+      <c r="H5" s="5">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="J5" s="5">
+        <v>7</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="F6" s="5">
         <v>1</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="J2" s="6">
+      <c r="G6" s="5">
+        <v>1</v>
+      </c>
+      <c r="H6" s="5">
+        <v>19000101</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="J6" s="5">
+        <v>1</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="F7" s="5">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="J7" s="5">
+        <v>5</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="F8" s="5">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5">
+        <v>1</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="J8" s="5">
+        <v>2</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="F9" s="5">
+        <v>1</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J9" s="5">
         <v>4</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K9" s="4" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B3" s="6" t="s">
+      <c r="D10" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="F3" s="6">
+      <c r="F10" s="4">
         <v>0</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G10" s="4">
         <v>0</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H10" s="5">
         <v>0</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="J3" s="6">
+      <c r="I10" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J10" s="5">
         <v>6</v>
       </c>
-      <c r="K3" s="5" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="K10" s="4" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="F4" s="6">
+      <c r="D11" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F11" s="4">
         <v>0</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G11" s="4">
         <v>0</v>
       </c>
-      <c r="H4" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="J4" s="6">
+      <c r="H11" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J11" s="5">
         <v>3</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K11" s="4" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="D12" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="F5" s="6">
+      <c r="F12" s="4">
         <v>0</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="5">
+        <v>0</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J12" s="5">
+        <v>7</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="F13" s="5">
         <v>1</v>
       </c>
-      <c r="H5" s="6">
+      <c r="G13" s="4">
+        <v>1</v>
+      </c>
+      <c r="H13" s="5">
+        <v>19000101</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="J13" s="5">
+        <v>1</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="F14" s="4">
         <v>0</v>
       </c>
-      <c r="I5" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="J5" s="6">
-        <v>7</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="F6" s="6">
+      <c r="G14" s="4">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5">
+        <v>0</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J14" s="5">
+        <v>5</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F15" s="5">
         <v>1</v>
       </c>
-      <c r="G6" s="6">
-        <v>1</v>
-      </c>
-      <c r="H6" s="6">
-        <v>19000101</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="J6" s="6">
-        <v>1</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="F7" s="6">
+      <c r="G15" s="4">
         <v>0</v>
       </c>
-      <c r="G7" s="6">
-        <v>1</v>
-      </c>
-      <c r="H7" s="6">
-        <v>0</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="J7" s="6">
-        <v>5</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="F8" s="6">
-        <v>1</v>
-      </c>
-      <c r="G8" s="6">
-        <v>1</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="J8" s="6">
+      <c r="H15" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J15" s="5">
         <v>2</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="K15" s="4" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="F9" s="6">
-        <v>1</v>
-      </c>
-      <c r="G9" s="5">
-        <v>0</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="J9" s="6">
-        <v>4</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="F10" s="5">
-        <v>0</v>
-      </c>
-      <c r="G10" s="5">
-        <v>0</v>
-      </c>
-      <c r="H10" s="6">
-        <v>0</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="J10" s="6">
-        <v>6</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="F11" s="5">
-        <v>0</v>
-      </c>
-      <c r="G11" s="5">
-        <v>0</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="J11" s="6">
-        <v>3</v>
-      </c>
-      <c r="K11" s="5" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="F12" s="5">
-        <v>0</v>
-      </c>
-      <c r="G12" s="5">
-        <v>0</v>
-      </c>
-      <c r="H12" s="6">
-        <v>0</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="J12" s="6">
-        <v>7</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="F13" s="6">
-        <v>1</v>
-      </c>
-      <c r="G13" s="5">
-        <v>1</v>
-      </c>
-      <c r="H13" s="6">
-        <v>19000101</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="J13" s="6">
-        <v>1</v>
-      </c>
-      <c r="K13" s="5" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="F14" s="5">
-        <v>0</v>
-      </c>
-      <c r="G14" s="5">
-        <v>0</v>
-      </c>
-      <c r="H14" s="6">
-        <v>0</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="J14" s="6">
-        <v>5</v>
-      </c>
-      <c r="K14" s="5" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="F15" s="6">
-        <v>1</v>
-      </c>
-      <c r="G15" s="5">
-        <v>0</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="J15" s="6">
-        <v>2</v>
-      </c>
-      <c r="K15" s="5" t="s">
-        <v>274</v>
-      </c>
-    </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B22" s="3"/>
+      <c r="B22" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K22" xr:uid="{00000000-0001-0000-0200-000000000000}"/>

</xml_diff>